<commit_message>
new metrics + getting tags
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U57"/>
+  <dimension ref="A1:X57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,70 +466,85 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>model_filters</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>answer</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>user_mark</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>contexts</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>sentence_count</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>word_count</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>avg_sentence_len</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>unique_word_ratio</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>faithfulness_score_entailment</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>faithfulness_score_neutral</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>faithfulness_score_contradiction</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>answer_correctness_literal</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>answer_correctness_neural</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>answer_relevance</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>jaccard_similarity</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>cosine_tag_answer</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>response_time</t>
         </is>
@@ -573,48 +588,59 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>Рейтинги студентов в НИУ ВШЭ позволяют оценить их успехи в освоении дисциплин. Текущий рейтинг сравнивает образовательные результаты студентов за полугодие, а кумулятивный включает результаты после пересдач. Рейтинги влияют на принятие управленческих решений и помогают в оценке качества и результативности обучения. Результаты рейтингов доступны в личном кабинете на портале НИУ ВШЭ или в LMS (Learning management system) после входа по логину и паролю от корпоративной почты. Если результаты неверны, студенты могут обратиться в учебный офис с заявлением об ошибке в течение двух рабочих дней.  Подробнее: https://www.hse.ru/evaluation/instructors\_access https://www.hse.ru/studyspravka/rate</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>али преподаватели, принимавшие экзамены. Рассчитывается таблица автоматически по единым принципам для всех факультетов и филиалов НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики). Так как в этом процессе есть "ручной" участок, то вероятны технические ошибки. Поэтому рейтинговые таблицы в определенные сроки предъявляются студентам и, если студент обнаружил неточности (не те оценки, не те дисциплины) он имеет возможность в течение двух рабочих дней заявить об обнаруженной ошибке в учебный офис. Документы Положение о рейтинговой системе комплексной оценки знаний студентов образовательных программ бакалавриата, специалитета и магистратуры Национального исследовательского университета «Высшая школа экономики»Получение доступа коценкам_ Получение доступа к оценкам Как узнать свои результаты? Собственные результаты преподавателя, начиная с результатов за 2019–2020 учебный год, доступны в его личном кабинете в LMS (Learning management system) (с возможностью прямого перехода из Единого личного кабинета). Старые результаты (за 2017–1018 и 2018–2019 год) доступны в личном кабинете на портале НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики). В личный кабинет LMS (Learning management system) вы можете зайти по логину и паролю от корпоративной почты по ссылке https://lms.hse.ru/ , нажав кнопку «Войти через ЕЛК». Если зайти через ЕЛК (единый личный кабинет) не получается и вы видите в LMS (Learning management system) сообщение «User not found», то обратитесь по ссылке . В Единый личный кабинет вы можете зайти по логину и паролю от корпоративной почты по ссылке https://lk.hse.ru/ . Если зайти в ЕЛК (единый личный кабинет) не получается, обратитесь по ссылке . В личный кабинет на портале вы можете зайти по логину и паролю от корпоративной почты по ссылке http://www.hse.ru/user/ . Если у вас не</t>
         </is>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>6</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>84</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>14</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>0.7976190476190477</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>0.8945921063423157</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>0.01678583957254887</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>0.08862209320068359</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>28.70188653330036</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>0.681091845035553</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>0.436910480260849</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.3842901587486267</v>
+      </c>
+      <c r="X2" t="n">
         <v>4.300594</v>
       </c>
     </row>
@@ -656,48 +682,59 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Английский язык', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Социальные вопросы', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы?  Подробнее: https://nnov.hse.ru/aup/sdu/ https://www.hse.ru/studyspravka/kud</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>студентов равно двум — это значит, что у студента две задолженности, и он допускается к пересдачам, но если получит третью неудовлетворительную оценку, то будет отчислен. Критическое значение КУД (качество учебной деятельности) для студентов, относящихся к отдельным категориям равно пяти , если превышение обычного КУД (качество учебной деятельности) в отношении студента зафиксировано в первый раз . Студенты, КУД (качество учебной деятельности) которых превышает критическое значение (с учетом отнесения студента к отдельной категории и наличия или отсутствия повтора критической ситуации), подлежат отчислению как не выполняющие обязанности по добросовестному освоению образовательной программы и выполнению учебного плана. Подробнее об отдельных категориях студентов . Пример расчета обычного КУД (качество учебной деятельности) : КУД=0 — у студента нет задолженностей, все хорошо КУД=2 — у студента две задолженности, он допускается к пересдачам КУД=4 — у студента четыре задолженности, он подлежит отчислению Документы Положение об организации промежуточной аттестации и текущего контроля успеваемости студентов НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) (ПО</t>
         </is>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>4</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>22</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>5.5</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>0.9545454545454546</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>0.5484193563461304</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>0.2526068091392517</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>0.1989738792181015</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>6.586810189291431</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>0.4471128880977631</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>0.5040789842605591</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.3524247407913208</v>
+      </c>
+      <c r="X3" t="n">
         <v>2.787384</v>
       </c>
     </row>
@@ -739,48 +776,59 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>Обратная связь от студентов является важной частью учебного процесса и помогает улучшить качество преподавания. В НИУ ВШЭ существует система студенческой оценки преподавания (СОП), где студенты могут оставить свои отзывы и предложения по улучшению работы преподавателей. Эти отзывы рассматриваются и учитываются при последующей реализации учебных курсов. Если у вас есть конкретные жалобы или предложения по работе преподавателя, вы можете оставить свои комментарии в соответствующем разделе СОП. Кроме того, вы можете обратиться напрямую к преподавателю или в учебный офис своей программы для обсуждения волнующих вас вопросов. Важно помнить, что конструктивная критика и аргументированные предложения помогают лучше понять потребности и ожидания студентов, что способствует дальнейшему развитию образовательного процесса.  Подробнее: http://www.hse.ru/evaluation/students\_mission https://www.hse.ru/evaluation/instructors\_goals https://www.hse.ru/evaluation/students\_structure https://www.hse.ru/evaluation/instructors\_techfaq</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>радикального изменения того или иного учебного курса при следующей его реализации. Обычно преподаватели получают оценки в течение пары недель после завершения учебного периода (включая сессию). Каждый год я просматриваю и анализирую баллы СОП (студенческая оценка преподавания), но гораздо внимательнее я смотрю на развернутые ответы и мнения студентов. Именно они оказываются наиболее полезны для достраивания или перекройки учебного курса. При этом я стараюсь принимать во внимание частотность тех или иных мнений. Чем чаще отзыв, совет или пожелание повторяется, тем выше его ценность для меня и тем с большей вероятностью я приму решение что-либо поменять в своем курсе. На единичные негативные отзывы я смотрю серьезно, только если в них есть хотя бы какие-либо аргументы. Если студент просто пишет, что ему «не понравились лекции», и не объясняет почему, доверия к такому отзыву в разы меньше. В конце концов, в университете мы учим аргументировать свою позицию и обосновывать свои суждения, даже если они носят оценочный характер. Вдовин Алексей Владимирович Школа филологических наук: Доцент (из материала для университетского издания « Окна роста » ) Почти все отзывы так или иначе полезны. Одни упоминают о конкретныхиторией Возможность внеаудиторного общения по учебным и научным вопросам Открытые вопросы (развернутый ответ): Что вам нравится в работе данного преподавателя (успешные практики и форматы, стиль взаимодействия и др.) Что бы вы предложили изменить в работе данного преподавателя (чего не хватает, что кажется лишним и т.д.) Советы по заполнению обратной связи по преподавателям 1\\. Вспомните все форматы, в которых преподаватель с вами работал . Как и с дисциплинами, впечатление о преподавателе тоже часто составляется на основе одного случая — например, после написания контрольной или общения по почте. Однако работа преподавателя гораздо шире — она включает в себя и проведение занятий, и объяснение заданий, и возможность поговорить о теме курсовой или ВКР (выпускная квалификационная работа), и выставление оценок. Если вы прокомментируете все виды вашей работы с преподавателем, отзыв получится объективнее, а преподаватель поймёт, над чем можно поработать. 2\\. Оцените эксперименты, которые проводит преподаватель . Курсы в Вышке меняются каждый год — преподаватели вводят новые темы занятий, обновляют презентации и форматы работы, вводят практические блоки. И им важно знать вашу реакцию на новые форматы работы — поэтому не стесняйтесь говоритьПомощь спроблемами_ Помощь с проблемами В данных замечены ошибки или неточности: чего-то не хватает или что-то лишнее Отправьте заявку с изложением проблемы по ссылке или письмом на rating@hse.ru . Нет доступа к результатам, а они нужны очень срочно Напишите менеджеру департамента, школы или кафедры, где вы работаете или где ранее преподавали (и к чему относятся те результаты, которые срочно нужны), и попросите прислать результаты СОП (студенческая оценка преподавания) выгрузкой в виде файла. Если от них нет ответа, напишите с аналогичной просьбой на rating@hse.ru , переслав переписку. Иная проблема с результатами Оставьте заявку по ссылке или напишите письмо на rating@hse.ru . пользоваться, и так далее. А каждый год число таких полезных отзывов растёт: в 2022 году студенты оставили более 20 тысяч открытых комментариев об учебном процессе в целом. Дирекция основных образовательных программ тщательно следит за обратной связью студентов в СОП (студенческая оценка преподавания) по организации учебного процесса. Мы используем комментарии для того, чтобы улучшать сервисы, работающие на весь университет — например, процедуру выбора майноров и МАГОЛЕГО. Так, в 2022 году студенты столкнулись с рядом технических и организационных проблем при выборе факультативов и курсов по выбору, и мы в Центре сервиса « Траектория » , провели анализ данных СОП (студенческая оценка преподавания), чтобы понять, какие именно сложности в поиске и выборе курсов для формировании своей траектории встречались чаще всего — и суметь их разрешить. Чичик Наталья Вячеславовна Центр сервиса «Траектория»: Руководитель центра</t>
         </is>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>7</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>106</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>15.14285714285714</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>0.8018867924528302</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>0.9558947086334229</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>0.01458257716149092</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>0.02952262386679649</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>17.12786091703714</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>0.6304216384887695</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>0.4062119424343109</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.3034822344779968</v>
+      </c>
+      <c r="X4" t="n">
         <v>4.460494</v>
       </c>
     </row>
@@ -822,44 +870,55 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Деньги', 'Другое', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Английский язык', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Социальные вопросы', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы? _ В своем ответе я больше опирался на свои знания, чем на документы НИУ ВШЭ. Вероятно, тема запроса не соответствует моим функциям или мне стоит еще поучиться! Может ты уточнишь свой вопрос?_</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="n">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
         <v>7</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>54</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>7.714285714285714</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>0.8888888888888888</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>0.1772089004516602</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>0.7732542753219604</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>0.04953683540225029</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>0</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>0.03415575623512268</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>0.3118091225624084</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
+        <v>0.07692307692307693</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.3378399908542633</v>
+      </c>
+      <c r="X5" t="n">
         <v>21.088965</v>
       </c>
     </row>
@@ -901,48 +960,59 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>Ваши оценки доступны в вашем личном кабинете в LMS (Learning management system) или на портале НИУ ВШЭ. Вы можете войти в личный кабинет с использованием логина и пароля от корпоративной почты. Если у вас возникают проблемы с доступом, рекомендуется обратиться за помощью.  Подробнее: https://nnov.hse.ru/aup/sdu/ https://www.hse.ru/evaluation/instructors\_goals https://www.hse.ru/evaluation/students\_structure https://www.hse.ru/evaluation/instructors\_access</t>
         </is>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>радикального изменения того или иного учебного курса при следующей его реализации. Обычно преподаватели получают оценки в течение пары недель после завершения учебного периода (включая сессию). Каждый год я просматриваю и анализирую баллы СОП (студенческая оценка преподавания), но гораздо внимательнее я смотрю на развернутые ответы и мнения студентов. Именно они оказываются наиболее полезны для достраивания или перекройки учебного курса. При этом я стараюсь принимать во внимание частотность тех или иных мнений. Чем чаще отзыв, совет или пожелание повторяется, тем выше его ценность для меня и тем с большей вероятностью я приму решение что-либо поменять в своем курсе. На единичные негативные отзывы я смотрю серьезно, только если в них есть хотя бы какие-либо аргументы. Если студент просто пишет, что ему «не понравились лекции», и не объясняет почему, доверия к такому отзыву в разы меньше. В конце концов, в университете мы учим аргументировать свою позицию и обосновывать свои суждения, даже если они носят оценочный характер. Вдовин Алексей Владимирович Школа филологических наук: Доцент (из материала для университетского издания « Окна роста » ) Почти все отзывы так или иначе полезны. Одни упоминают о конкретных Вопросы по проектам Числовые оценки (от 1 до 5 + « затрудняюсь ответить » ): Полезность проекта для вашей будущей карьеры Полезность проекта для расширения кругозора и разностороннего развития Новизна полученных на проекте знаний и навыков Качество организации проекта со стороны руководителя Сложность проекта для успешного прохождения («1» — проект очень легкий, «5» — проект очень сложный для прохождения) Открытые вопросы (развернутый ответ): Замечания и предложения относительно организации данного проекта Советы по заполнению обратной связи по проектам 1\\. Оцените, как проект помог вам в освоении образовательной программы или индивидуального учебного плана . Проекты бывают разные, но они всегда развивают какие-то навыки — прикладные или исследовательские. Мы рекомендуем вам оценить не только то, как проект помог вам развить новые умения, но и то, как эти умения работают в связке с курсами и проектами вашей образовательной программы 2\\. Расскажите о самом процессе проектной работы . Для проекта важны не только полученные навыки и итоговый продукт — зачастую очень важны и атмосфера в команде, и качество материалов, которые вам давали для обучения, и грамотность постановки задач. Поэтому старайтесь вспоминать о внутренних аспектах организации проекта,Получение доступа коценкам_ Получение доступа к оценкам Как узнать свои результаты? Собственные результаты преподавателя, начиная с результатов за 2019–2020 учебный год, доступны в его личном кабинете в LMS (Learning management system) (с возможностью прямого перехода из Единого личного кабинета). Старые результаты (за 2017–1018 и 2018–2019 год) доступны в личном кабинете на портале НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики). В личный кабинет LMS (Learning management system) вы можете зайти по логину и паролю от корпоративной почты по ссылке https://lms.hse.ru/ , нажав кнопку «Войти через ЕЛК». Если зайти через ЕЛК (единый личный кабинет) не получается и вы видите в LMS (Learning management system) сообщение «User not found», то обратитесь по ссылке . В Единый личный кабинет вы можете зайти по логину и паролю от корпоративной почты по ссылке https://lk.hse.ru/ . Если зайти в ЕЛК (единый личный кабинет) не получается, обратитесь по ссылке . В личный кабинет на портале вы можете зайти по логину и паролю от корпоративной почты по ссылке http://www.hse.ru/user/ . Если у вас не</t>
         </is>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>4</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>43</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>10.75</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>0.9302325581395349</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>0.9036950469017029</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>0.01110771112143993</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>0.08519726246595383</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>10.95393089990464</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>0.6199450492858887</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>0.2405778020620346</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.371463805437088</v>
+      </c>
+      <c r="X6" t="n">
         <v>3.440407</v>
       </c>
     </row>
@@ -984,48 +1054,59 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>['Внеучебка', 'Другое', 'Внеучебка', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>В НИУ ВШЭ существуют различные внеучебные клубы, такие как Студенческий Совет, Центр оперативной помощи, Социальный комитет, Правовой комитет, Совет иностранных студентов, Комитет медиакоммуникаций и другие. Эти организации занимаются различными вопросами и проблемами студентов, включая защиту прав, улучшение качества образования и предоставление социальной помощи. Более подробную информацию о каждом из них можно получить на сайте университета.  Подробнее: https://www.hse.ru/studyspravka/edmodel\_bachelor\_20 https://nnov.hse.ru/nnovstudents/student\_council</t>
         </is>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>образования решит данный вопрос! И это еще малая часть того, что входит в компетенцию СС. Листай вниз и становись еще ближе к нам! Студсовет НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) - НН – выборный представительный орган нашего университета. Через него мы, студенты, можем отстаивать свои интересы, права и получать различные рекомендации и консультации. В Студсовете вы научитесь лучше понимать людей, их мотивы, мнения и действия. Каждый из вас может делать жизни студентов лучше! Не только помогать, но и обсуждать, улучшать, воздействовать на те процессы, которые кажутся независимыми и не поддающимися изменениям. Илья Шалявин Председатель Дмитрий Цирулев Секретарь Студсовета Егор Батяев Глава Комитета по качеству образования Екатерина Портная Глава Социального комитета Эстер Гейн Глава Комитета медиакомуникаций Али Имран Председатель Совета иностранных студентов Дарья Ромащёва Глава HR отдела Сообщество Студенческого Совета</t>
         </is>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>4</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>56</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>14</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>0.875</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>0.6234458684921265</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>0.2694630026817322</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>0.1070911213755608</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>24.65371947617363</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>0.5859071016311646</v>
       </c>
-      <c r="T7" t="n">
+      <c r="U7" t="n">
         <v>0.3031834363937378</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0.2170685827732086</v>
+      </c>
+      <c r="X7" t="n">
         <v>3.602912</v>
       </c>
     </row>
@@ -1067,44 +1148,55 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы? _ В своем ответе я больше опирался на свои знания, чем на документы НИУ ВШЭ. Вероятно, тема запроса не соответствует моим функциям или мне стоит еще поучиться! Может ты уточнишь свой вопрос?_</t>
         </is>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>-1</v>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="n">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
         <v>7</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>54</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>7.714285714285714</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>0.8888888888888888</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>0.1772089004516602</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>0.7732542753219604</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>0.04953683540225029</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>0</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>0.03415575623512268</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>0.4769177436828613</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.4006629586219788</v>
+      </c>
+      <c r="X8" t="n">
         <v>21.213023</v>
       </c>
     </row>
@@ -1146,48 +1238,59 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы? _ В своем ответе я больше опирался на свои знания, чем на документы НИУ ВШЭ. Вероятно, тема запроса не соответствует моим функциям или мне стоит еще поучиться! Может ты уточнишь свой вопрос?_</t>
         </is>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>-1</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Прочие платежи за услуги Прочие платежи за услуги (НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Пермь) Internet Explorer ниже 9 версии не поддерживается. Используйте более современную версию браузера или Google Chrome или Mozilla Firefox Внимание! В данном разделе запрещено осуществлять возврат средств по оплате труда и стипендиям! Способы оплаты Банковская карта / SberPay К оплате принимаются карты платежных систем МИР, Visa и Mastercard Фамилия Имя Отчество: Фамилия Имя Отчество * Адрес электронной почты: Адрес электронной почты * Телефон: Телефон Код подразделения: Код подразделения * Номер договора: Номер договора ID договора: ID договора Назначение платежа: Назначение платежа * НДС: Включает НДС Без НДС Сумма: Сумма * руб. коп. Далее или Исправить * – Поле обязательно для заполнения.Пожертвования Высшая школа экономики стала для многих символом качественного образования, высоких стандартов исследовательской работы, лабораторией инновационных идей и проектов. Мы живём в соответствии с понятными всем ценностями и готовы следовать им при любых внешних обстоятельствах. Мы научились зарабатывать на рынке и разумно вкладывать средства так, чтобы обеспечить постоянный рост, в том числе за счёт привлечения лучших преподавателей и учёных, высокопрофессиональных менеджеров и вдохновляющих лидеров. Вышка – амбициозный университет, находящийся в постоянном развитии. Сейчас нашей глобальной целью является закрепление позиции флагмана российского образования и получение международного признания в приоритетных областях научного знания. Достижение такой высокой цели невозможно без доверия и поддержки со стороны широкого сообщества, его выпускников, друзей и партнёров. С вашим участием мы можем сделать больше!</t>
         </is>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>7</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>54</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>7.714285714285714</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>0.8888888888888888</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>0.5413159728050232</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>0.3722324073314667</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>0.08645159751176834</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>9.713934232580728</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>0.529745876789093</v>
       </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>0.4769177436828613</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.4006629586219788</v>
+      </c>
+      <c r="X9" t="n">
         <v>2.728583</v>
       </c>
     </row>
@@ -1229,48 +1332,59 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Английский язык', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Другое', 'Деньги', 'Другое', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Английский язык', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование']</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>Что-то в вашем вопросе меня смущает. Может, поговорим на другую тему?  Подробнее: https://www.hse.ru/studyspravka/edmodel\_bachelor\_20 https://www.hse.ru/evaluation/instructors\_access https://www.hse.ru/studyspravka/kud https://www.hse.ru/studyspravka/ras\_stud</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>-1</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Получение доступа коценкам_ Получение доступа к оценкам Как узнать свои результаты? Собственные результаты преподавателя, начиная с результатов за 2019–2020 учебный год, доступны в его личном кабинете в LMS (Learning management system) (с возможностью прямого перехода из Единого личного кабинета). Старые результаты (за 2017–1018 и 2018–2019 год) доступны в личном кабинете на портале НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики). В личный кабинет LMS (Learning management system) вы можете зайти по логину и паролю от корпоративной почты по ссылке https://lms.hse.ru/ , нажав кнопку «Войти через ЕЛК». Если зайти через ЕЛК (единый личный кабинет) не получается и вы видите в LMS (Learning management system) сообщение «User not found», то обратитесь по ссылке . В Единый личный кабинет вы можете зайти по логину и паролю от корпоративной почты по ссылке https://lk.hse.ru/ . Если зайти в ЕЛК (единый личный кабинет) не получается, обратитесь по ссылке . В личный кабинет на портале вы можете зайти по логину и паролю от корпоративной почты по ссылке http://www.hse.ru/user/ . Если у вас неит отчислению Документы Положение об организации промежуточной аттестации и текущего контроля успеваемости студентов НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) (ПОПАТКУС (Положения о промежуточной аттестации и текущем контроле успеваемости студентов)) Полезные ссылки Электронная зачетная книжка LMS (Learning management system) Контроль знаний студентов Шкала соответствия оценок Перенос второй пересдачи дисциплины Отчисление Восстановление с местоположением корпуса, где запланировано занятие; интегрировать занятия в личный календарь. Если обнаружен конфликт в расписании Дисциплин учебного плана : можно либо перевестись в другую учебную группу в рамках одной дисциплины, либо, если группа только одна, можно заменить одну из вариативных дисциплин на другую, с более подходящим расписанием — обратитесь к менеджеру своей образовательной программы за консультацией. Экзаменов на сессии : если в расписании сессии в день стоит несколько экзаменов (включая повторные сдачи блокирующих в течение 10 дней до сессии), то можно либо сдавать несколько экзаменов в один день, если по времени не пересекаются (в этом случае нельзя апеллировать к процедуре экзамена), либо подать заявку о переносе одного из экзаменов на другое время не позднее трех дней до начала сессии. Пересдач с расписанием занятий : подайте заявку для изменения имеющейся даты пересдачи не позднее трех дней до начала периода пересдач по графику учебного процесса . Если возникли проблемы с расписанием Если в расписании с использованием любого из сервисов не отображаются некоторые занятия, отсутствует расписание по некоторым дисциплинам, или не прикреплены ссылки к онлайн-занятиям, необходимо обратиться в учебный офис вашей образовательной программы — контак которые он может выбирать для изучения. Подробнее про ИУП (индивидуальный учебный план) Полезные ссылки Центр сервиса "Траектория" Выбор курсов ДОЦ Майноры Практическая подготовка Английский язык Цифровые компетенции (Data Culture) ГИА (государственная итоговая аттестация)</t>
         </is>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>3</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>13</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>4.333333333333333</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>1</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>0.8971853852272034</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>0.01814925856888294</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>0.08466531336307526</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>4.438591048861381</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>0.4992415904998779</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>0.5054616928100586</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
+        <v>0.07692307692307693</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.4734145402908325</v>
+      </c>
+      <c r="X10" t="n">
         <v>3.095392</v>
       </c>
     </row>
@@ -1312,48 +1426,59 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
+          <t>['Деньги', 'Другое', 'Учебный процесс', 'ГИА', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Социальные вопросы', 'ОВЗ', 'Выпускникам', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Социальные вопросы', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
           <t>Как у нейросетевой языковой модели у меня не может быть настроения, но почему-то я совсем не хочу говорить на эту тему.  Подробнее: https://www.hse.ru/scholarships/social\_scholarship\_new https://www.hse.ru/studyspravka/russian https://studentcentre.hse.ru/ https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>-1</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>ES ). Подать заявку выпускнику Для подачи заявки необходимо авторизоваться в Едином личном кабинете. Если у Вас нет аккаунта в ЕЛК (единый личный кабинет), пожалуйста, зарегистрируйтесь по ссылке Проверить подлинность диплома гос.образца в реестре Рособрнадзора (ФИС ФРДО) Проверка подлинности диплома государственного образца осуществляется на сайте Рособрнадзора ( ФИС ФРДО ). Дипломы выпускников - граждан РФ 2021 года выпуска и позднее передаются в ФИС ФРДО только при условии предоставления СНИЛС. Выпускники, получившие дипломы в 2021 году и позднее и представившие на момент выпуска данные СНИЛС, могут проверить свой диплом на портале Госуслуг . В случае, если Вы не нашли свой диплом в ФИС ФРДО , сообщите нам об этом по электронной почте . Проверить подлинность диплома собственного образца НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Сервисы для внешних пользователей Студентам других образовательных организаций консультируем по вопросам переводов из зарубежных университетов в НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) студентов, являющихся гражданами РФ, ДНР, ЛНРценно освоить всю образовательную программу. [1] Тестирование по русскому языку как иностранному языку (ТРКИ) основано на единой сертификационной системе определения уровня владения практическим русским языком и построено с учетом целей его использования, навыков и умений в употреблении языковых средств для реализации определенных тактик речевого поведения в основных видах речевой деятельности. Кому не нужно изучать дисциплины по русскому языку? Изучать дисциплины по русскому языку не требуется иностранным студентам, которые могут документально подтвердить свой уровень владения русским языком. Для этого необходимо подать электронное заявление в Центр сервиса Студент. Те студенты, заявления которых будут одобрены, освобождаются от прохождения входного тестирования и обязательного изучения русского языка. Если студент владеет русским языком на необходимом уровне, но не может подтвердить этот уровень документально, он может подать заявление о прохождении тестирования (независимого экзамена, а при отсутствии по техническим причинам такой возможности – его эквивалента), по результатам которого может быть так же освобожден от обязательного прохождения языковой подготовки. Какими документами можно подтвердить уровень владения русским языком? Для подтверждения уровня владения русским языком через электронное заявление в Центр сервиса Студент принимаются следующие документы. Иностранные граждане и лица без гражданства, имеющие право на перевод с платного обучения на бесплатное Студенты НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) - иностранные граждане и лица без гражданства, имеющие право на перевод с платного обучения на бесплатное Основание Гражданство (либо статус лица гражданства) Условие Документы, подтверждающие соответствующий статус 1 Соглашение о сотрудничестве в области образования, г. Ташкент, 15 мая 1992 г. Азербайджан, Армения, Беларусь, Казахстан, Кыргызстан, Молдова, Таджикистан, Туркменистан, Узбекистан, Украина Наличие гражданства страны- участницы соглашения Наличие у иностранного гражданина вида на жительство в Российской Федерации 2 Соглашение между Правительством Российской Федерации и Правительством Республики Грузия о сотрудничестве в области культуры, науки и образования от 2 февраля 1994 г. № 49 Грузия Наличие гражданства страны- участницы соглашения Наличие у иностранного гражданина вида на жительство в Российской Федерации 3 Соглашение между Правительством Российской Федерации и Правительством Республики Абхазия о сотрудничестве в области образования от 27.04.2012 ВНИМАНИЕ! Перечень направ В течение учебного года по предоставлению оригиналов документов в ЦСиБП (Архангельской О.В., Папуше Е.С.) и размещения копий документов в системе LMS (Learning management system). Документы принимаются в течение всего учебного года в системе LMS (Learning management system). На какой период времени назначается Назначается с даты подачи заявки (пакета документов) на социальную стипендию в LMS (Learning management system) до даты окончания действия подтверждающего документа (или отчисления студента). Оригиналы должны быть предоставлены в ЦСиБП по адресу Покровский бульвар,11, комната L105 (Архангельской О.В., Папуше Е.С.) По справке о получении (назначении) государственной социальной помощи по месту жительства стипендия назначается с даты подачи заявки (пакета документов) на социальную стипендию в LMS (Learning management system) (оригиналы - в ЦСиБП) на год с даты назначения государственной социальной помощ и. Процедура подачи заявки на конкурс/порядок назначения стипендии без конкурса Документы (оригиналы документов, подтверждающий социальный статус (справка, свидетельство, удостоверение) передаются в ЦСиБП (Архангельской О.В., Папуше Е.С.) в</t>
         </is>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>2</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>23</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>11.5</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>0.9130434782608695</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>0.6896648406982422</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>0.04020758345723152</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>0.2701276242733002</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>2.580729318503379</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>0.4536304771900177</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>0.5080456733703613</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.5291953682899475</v>
+      </c>
+      <c r="X11" t="n">
         <v>2.890775</v>
       </c>
     </row>
@@ -1395,48 +1520,59 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
           <t>Что-то в вашем вопросе меня смущает. Может, поговорим на другую тему?  Подробнее: https://nnov.hse.ru/aup/sdu/ https://www.hse.ru/studyspravka/russian https://www.hse.ru/studyspravka/rate https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>1</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>языке можно не переводить (оставить на языке оригинала), но желательно перевести название города/штата/провинции/страны. Нашли опечатку ? Выделите её, нажмите Ctrl+Enter и отправьте нам уведомление. Спасибо за участие! Сервис предназначен только для отправки сообщений об орфографических и пунктуационных ошибках.Социальные стипендии Студентам Материальная помощь Пособие по беременности и родам студентам Программа РЖД Бонус Стипендии Сотрудникам Материальная помощь Социальная поддержка сотрудников с инвалидностью Полное государственное обеспечение и доп.гарантии по социальной поддержке сирот Медицинское обслуживание ДМС для сотрудников Доврачебная медицинская помощь Предварительные и периодические медосмотры Медосмотр для конкурса ППС "Единое окно" по поддержке молодых семей информация о реализации "единого окна" от Минобрнауки России Федеральные меры поддержки Пособие по беременности и родам студентам Материальная поддержка студентов, имеющих детей Психологическая помощь Студенческое правовое бюро (юридическая помощь) Психологическая помощь и телефоны горячих линий Записаться на консультацию к психологу или коучу Государственные жилищные сертификаты — молодым ученым, в открытом доступе на сайтах образовательных программ в разделе Студентам - Рейтинги. На что влияет место в рейтинге Рейтинговая позиция часто используется для распределения различных студенческих благ. Студентам, которые оплачивают свое обучение, хорошее место в рейтинге может принести скидку на оплату обучения . Место в рейтинге может повлиять на возможность записаться на популярные дисциплины по выбору, майноры, общеуниверситетские факультативы . При принятии решения о выделении студенту гранта на академическую международную мобильность , также важную роль может сыграть ваш рейтинг. Как рассчитывается рейтинг Рейтинг определяется следующим образом: Каждый факультет принимает решение какие студенты будут друг с другом сравниваться. Возможно сравнение студентов одного курса одной образовательной программы, либо нескольких образовательных программ Для каждого студента определяется сумма произведений оценок на кредитный вес элемента учебного плана. Например, студент в течение полугодия изучал английский язык (4 кредита), математический анализ (5 кредитов) и историю (3 кредита). Получил по ним такие оценки: 8, 7, 10. Для этого студента рассчитывается показатель: 4*8+5*7+3*10 = 97. Так как у каждого студента Вышки учебный план индивидуальный, то, чем старше курс, тем разнообразнее набор</t>
         </is>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>3</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>13</v>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>4.333333333333333</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>1</v>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>0.9102593660354614</v>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>0.03921904042363167</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>0.05052163824439049</v>
       </c>
-      <c r="R12" t="n">
+      <c r="S12" t="n">
         <v>2.156214446938086</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>0.4362529516220093</v>
       </c>
-      <c r="T12" t="n">
+      <c r="U12" t="n">
         <v>0.5721657276153564</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.441891074180603</v>
+      </c>
+      <c r="X12" t="n">
         <v>2.622681</v>
       </c>
     </row>
@@ -1478,48 +1614,59 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
+          <t>['Деньги', 'Другое', 'Учебный процесс', 'ГИА', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Социальные вопросы', 'ОВЗ', 'Выпускникам', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Социальные вопросы', 'Другое', 'Деньги', 'Другое', 'Учебный процесс', 'ГИА', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Социальные вопросы', 'ОВЗ', 'Выпускникам', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
           <t>Как у нейросетевой языковой модели у меня не может быть настроения, но почему-то я совсем не хочу говорить на эту тему.  Подробнее: https://www.hse.ru/scholarships/social\_scholarship\_new https://www.hse.ru/studyspravka/russian https://studentcentre.hse.ru/ https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>-1</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>ES ). Подать заявку выпускнику Для подачи заявки необходимо авторизоваться в Едином личном кабинете. Если у Вас нет аккаунта в ЕЛК (единый личный кабинет), пожалуйста, зарегистрируйтесь по ссылке Проверить подлинность диплома гос.образца в реестре Рособрнадзора (ФИС ФРДО) Проверка подлинности диплома государственного образца осуществляется на сайте Рособрнадзора ( ФИС ФРДО ). Дипломы выпускников - граждан РФ 2021 года выпуска и позднее передаются в ФИС ФРДО только при условии предоставления СНИЛС. Выпускники, получившие дипломы в 2021 году и позднее и представившие на момент выпуска данные СНИЛС, могут проверить свой диплом на портале Госуслуг . В случае, если Вы не нашли свой диплом в ФИС ФРДО , сообщите нам об этом по электронной почте . Проверить подлинность диплома собственного образца НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Сервисы для внешних пользователей Студентам других образовательных организаций консультируем по вопросам переводов из зарубежных университетов в НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) студентов, являющихся гражданами РФ, ДНР, ЛНРценно освоить всю образовательную программу. [1] Тестирование по русскому языку как иностранному языку (ТРКИ) основано на единой сертификационной системе определения уровня владения практическим русским языком и построено с учетом целей его использования, навыков и умений в употреблении языковых средств для реализации определенных тактик речевого поведения в основных видах речевой деятельности. Кому не нужно изучать дисциплины по русскому языку? Изучать дисциплины по русскому языку не требуется иностранным студентам, которые могут документально подтвердить свой уровень владения русским языком. Для этого необходимо подать электронное заявление в Центр сервиса Студент. Те студенты, заявления которых будут одобрены, освобождаются от прохождения входного тестирования и обязательного изучения русского языка. Если студент владеет русским языком на необходимом уровне, но не может подтвердить этот уровень документально, он может подать заявление о прохождении тестирования (независимого экзамена, а при отсутствии по техническим причинам такой возможности – его эквивалента), по результатам которого может быть так же освобожден от обязательного прохождения языковой подготовки. Какими документами можно подтвердить уровень владения русским языком? Для подтверждения уровня владения русским языком через электронное заявление в Центр сервиса Студент принимаются следующие документы. Иностранные граждане и лица без гражданства, имеющие право на перевод с платного обучения на бесплатное Студенты НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) - иностранные граждане и лица без гражданства, имеющие право на перевод с платного обучения на бесплатное Основание Гражданство (либо статус лица гражданства) Условие Документы, подтверждающие соответствующий статус 1 Соглашение о сотрудничестве в области образования, г. Ташкент, 15 мая 1992 г. Азербайджан, Армения, Беларусь, Казахстан, Кыргызстан, Молдова, Таджикистан, Туркменистан, Узбекистан, Украина Наличие гражданства страны- участницы соглашения Наличие у иностранного гражданина вида на жительство в Российской Федерации 2 Соглашение между Правительством Российской Федерации и Правительством Республики Грузия о сотрудничестве в области культуры, науки и образования от 2 февраля 1994 г. № 49 Грузия Наличие гражданства страны- участницы соглашения Наличие у иностранного гражданина вида на жительство в Российской Федерации 3 Соглашение между Правительством Российской Федерации и Правительством Республики Абхазия о сотрудничестве в области образования от 27.04.2012 ВНИМАНИЕ! Перечень направ В течение учебного года по предоставлению оригиналов документов в ЦСиБП (Архангельской О.В., Папуше Е.С.) и размещения копий документов в системе LMS (Learning management system). Документы принимаются в течение всего учебного года в системе LMS (Learning management system). На какой период времени назначается Назначается с даты подачи заявки (пакета документов) на социальную стипендию в LMS (Learning management system) до даты окончания действия подтверждающего документа (или отчисления студента). Оригиналы должны быть предоставлены в ЦСиБП по адресу Покровский бульвар,11, комната L105 (Архангельской О.В., Папуше Е.С.) По справке о получении (назначении) государственной социальной помощи по месту жительства стипендия назначается с даты подачи заявки (пакета документов) на социальную стипендию в LMS (Learning management system) (оригиналы - в ЦСиБП) на год с даты назначения государственной социальной помощ и. Процедура подачи заявки на конкурс/порядок назначения стипендии без конкурса Документы (оригиналы документов, подтверждающий социальный статус (справка, свидетельство, удостоверение) передаются в ЦСиБП (Архангельской О.В., Папуше Е.С.) в ES ). Подать заявку выпускнику Для подачи заявки необходимо авторизоваться в Едином личном кабинете. Если у Вас нет аккаунта в ЕЛК (единый личный кабинет), пожалуйста, зарегистрируйтесь по ссылке Проверить подлинность диплома гос.образца в реестре Рособрнадзора (ФИС ФРДО) Проверка подлинности диплома государственного образца осуществляется на сайте Рособрнадзора ( ФИС ФРДО ). Дипломы выпускников - граждан РФ 2021 года выпуска и позднее передаются в ФИС ФРДО только при условии предоставления СНИЛС. Выпускники, получившие дипломы в 2021 году и позднее и представившие на момент выпуска данные СНИЛС, могут проверить свой диплом на портале Госуслуг . В случае, если Вы не нашли свой диплом в ФИС ФРДО , сообщите нам об этом по электронной почте . Проверить подлинность диплома собственного образца НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Сервисы для внешних пользователей Студентам других образовательных организаций консультируем по вопросам переводов из зарубежных университетов в НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) студентов, являющихся гражданами РФ, ДНР, ЛНРценно освоить всю образовательную программу. [1] Тестирование по русскому языку как иностранному языку (ТРКИ) основано на единой сертификационной системе определения уровня владения практическим русским языком и построено с учетом целей его использования, навыков и умений в употреблении языковых средств для реализации определенных тактик речевого поведения в основных видах речевой деятельности. Кому не нужно изучать дисциплины по русскому языку? Изучать дисциплины по русскому языку не требуется иностранным студентам, которые могут документально подтвердить свой уровень владения русским языком. Для этого необходимо подать электронное заявление в Центр сервиса Студент. Те студенты, заявления которых будут одобрены, освобождаются от прохождения входного тестирования и обязательного изучения русского языка. Если студент владеет русским языком на необходимом уровне, но не может подтвердить этот уровень документально, он может подать заявление о прохождении тестирования (независимого экзамена, а при отсутствии по техническим причинам такой возможности – его эквивалента), по результатам которого может быть так же освобожден от обязательного прохождения языковой подготовки. Какими документами можно подтвердить уровень владения русским языком? Для подтверждения уровня владения русским языком через электронное заявление в Центр сервиса Студент принимаются следующие документы</t>
         </is>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>2</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>23</v>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>11.5</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>0.9130434782608695</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>0.8664421439170837</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>0.01497307512909174</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>0.1185848340392113</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>1.738841246903425</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>0.45400670170784</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>0.5080456733703613</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
+        <v>0.07692307692307693</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.5291953682899475</v>
+      </c>
+      <c r="X13" t="n">
         <v>2.735338</v>
       </c>
     </row>
@@ -1561,48 +1708,59 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Другое', 'Учебный процесс', 'Социальные вопросы', 'ОВЗ', 'Другое', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Наука', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
           <t>Качество учебной деятельности (КУД) равно нулю (КУД=0) означает, что у вас нет задолженностей по дисциплинам, все оценки удовлетворительные. Это хороший показатель, который свидетельствует о успешном прохождении сессий.  Подробнее: https://www.hse.ru/studyspravka/practice https://nnov.hse.ru/aup/sdu/ https://www.hse.ru/studyspravka/zachetbook https://www.hse.ru/studyspravka/spec\_uslovia</t>
         </is>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>1</v>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>того, чтобы не были обесценены отзывы в Студенческой оценке преподавания . Оценки, полученные по промежуточной аттестации на сессии, а также оценки по всем элементам контроля, направляются преподавателем дисциплины студентам не позднее трех рабочих дней после определения оценок по промежуточной аттестации. Далее оценки передаются преподавателем в учебный офис не позднее пяти рабочих дней после окончания сессии. Что такое КУД (качество учебной деятельности) в зачетке и что он значит Простыми словами, показатель учебной деятельности (КУД (качество учебной деятельности)) — это количество дисциплин, по которым у студента есть неудовлетворительные оценки по итогам сессий. КУД=0 — у студента нет задолженностей, все хорошо КУД=2 — у студента две задолженности, он допускается к пересдачам, но если получит третью неудовлетворительную оценку, то будет отчислен КУД=3 и выше — у студента четыре задолженности, он подлежит отчислению Подробнее о КУД (качество учебной деятельности) Что делать, если обнаружена ошибка в расчете оценки Если студент обнаружил ошибки в расчете, то в течение пяти рабочих дней после получения доступа к файлу с расчетом промежуточной оценки необходимо обратиться к преподавателю, направив Вышке к отдельной категории обучающихся , что дает право таким обучающимся право на особые условия при освоении образовательной программы, а именно: на критическое значение КУД (качество учебной деятельности) равное пяти , если превышение обычного КУД (качество учебной деятельности) в отношении студента зафиксировано в первый раз; на возможность повторного изучения дисциплины один раз в течение всего периода обучения в Университете (за исключением случаев, когда академическая задолженность возникает в связи с невыбором темы курсовой работы) с сохранением текущих финансовых условий, до участия во второй пересдаче . работы по ЭПП (элемент практической подготовки) (при получении 1-2 кредитов за ЭПП (элемент практической подготовки) допустимо оценивание по шкале зачет / не зачет). в виде количества кредитов (применимо для любого ЭПП (элемент практической подготовки), кроме подготовки ВКР (выпускная квалификационная работа)), отражающих объем выполненной работы по ЭПП (элемент практической подготовки). Что это значит? Например, студент подписал задание на выполнение ЭПП (элемент практической подготовки), за которое максимум мог получить 5 кредитов. В результате он проделал весь отведенный ему объем работы, но качество данной работы оказалось низким. Тогда руководитель ЭПП (элемент практической подготовки) зачитывает ему все 5 кредитов, но за качество снижает оценку. Бывает и наоборот, студент подписал задание, но в итоге сделал гораздо меньше запланированного, зато на очень высоком уровне. Тогда вместо 5 кредитов руководитель ЭПП (элемент практической подготовки) выставляет ему, допустим, 2 кредита, зато ставит высокий балл за качество. Такая система применима к любым ЭПП (элемент практической подготовки), кроме подготовки ВКР (выпускная квалификационная работа), где количество кредитов строго закреплено учебным планом. Снижение</t>
         </is>
       </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
         <v>3</v>
       </c>
-      <c r="L14" t="n">
+      <c r="M14" t="n">
         <v>29</v>
       </c>
-      <c r="M14" t="n">
+      <c r="N14" t="n">
         <v>9.666666666666666</v>
       </c>
-      <c r="N14" t="n">
+      <c r="O14" t="n">
         <v>0.9655172413793104</v>
       </c>
-      <c r="O14" t="n">
+      <c r="P14" t="n">
         <v>0.6913638710975647</v>
       </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
         <v>0.05740376561880112</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="R14" t="n">
         <v>0.2512323260307312</v>
       </c>
-      <c r="R14" t="n">
+      <c r="S14" t="n">
         <v>7.918811153101803</v>
       </c>
-      <c r="S14" t="n">
+      <c r="T14" t="n">
         <v>0.5367180109024048</v>
       </c>
-      <c r="T14" t="n">
+      <c r="U14" t="n">
         <v>0.4451499581336975</v>
       </c>
-      <c r="U14" t="n">
+      <c r="V14" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.4815196096897125</v>
+      </c>
+      <c r="X14" t="n">
         <v>3.313501</v>
       </c>
     </row>
@@ -1644,44 +1802,55 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы?  Подробнее: https://www.hse.ru/scholarships/social\_scholarship\_new https://nnov.hse.ru/aup/sdu/ https://www.hse.ru/studyspravka/rate https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>-1</v>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="n">
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
         <v>4</v>
       </c>
-      <c r="L15" t="n">
+      <c r="M15" t="n">
         <v>22</v>
       </c>
-      <c r="M15" t="n">
+      <c r="N15" t="n">
         <v>5.5</v>
       </c>
-      <c r="N15" t="n">
+      <c r="O15" t="n">
         <v>0.9545454545454546</v>
       </c>
-      <c r="O15" t="n">
+      <c r="P15" t="n">
         <v>0.07461577653884888</v>
       </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
         <v>0.8679574131965637</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="R15" t="n">
         <v>0.05742685869336128</v>
       </c>
-      <c r="R15" t="n">
+      <c r="S15" t="n">
         <v>0</v>
       </c>
-      <c r="S15" t="n">
+      <c r="T15" t="n">
         <v>0.0785263255238533</v>
       </c>
-      <c r="T15" t="n">
+      <c r="U15" t="n">
         <v>0.5888119339942932</v>
       </c>
-      <c r="U15" t="n">
+      <c r="V15" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0.5203778743743896</v>
+      </c>
+      <c r="X15" t="n">
         <v>2.789608</v>
       </c>
     </row>
@@ -1723,44 +1892,55 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы?  Подробнее: https://www.hse.ru/scholarships/social\_scholarship\_new https://nnov.hse.ru/aup/sdu/ https://www.hse.ru/studyspravka/rate https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
         <v>-1</v>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="n">
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
         <v>4</v>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v>22</v>
       </c>
-      <c r="M16" t="n">
+      <c r="N16" t="n">
         <v>5.5</v>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>0.9545454545454546</v>
       </c>
-      <c r="O16" t="n">
+      <c r="P16" t="n">
         <v>0.07461577653884888</v>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>0.8679574131965637</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="R16" t="n">
         <v>0.05742685869336128</v>
       </c>
-      <c r="R16" t="n">
+      <c r="S16" t="n">
         <v>0</v>
       </c>
-      <c r="S16" t="n">
+      <c r="T16" t="n">
         <v>0.0785263255238533</v>
       </c>
-      <c r="T16" t="n">
+      <c r="U16" t="n">
         <v>0.5888119339942932</v>
       </c>
-      <c r="U16" t="n">
+      <c r="V16" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.5203778743743896</v>
+      </c>
+      <c r="X16" t="n">
         <v>2.752867</v>
       </c>
     </row>
@@ -1802,48 +1982,59 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Траектории обучения', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
           <t>Как у нейросетевой языковой модели у меня не может быть настроения, но почему-то я совсем не хочу говорить на эту тему.  Подробнее: https://www.hse.ru/studyspravka/Skidki https://nnov.hse.ru/aup/sdu/ https://www.hse.ru/studyspravka/perbud https://www.hse.ru/scholarships/rzd\_bonus</t>
         </is>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
         <v>-1</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>летней сессии, если их положение в рейтинге изменилось. Основания для лишения скидки Студент может быть лишен скидки: Любого вида - если ему объявлено дисциплинарное взыскание в виде выговора за нарушение Устава НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики), Правил внутреннего распорядка обучающихся НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики), Правил внутреннего распорядка общежития и иных локальных актов по вопросам организации и осуществления образовательной деятельности. Централизованной по результатам поступления на программы бакалавриата/специалитета (за исключением скидки по результатам вступительных испытаний) и магистратуры - при несоответствии студента одному или нескольким критериям успешного обучения, выразившееся в получении в предшествующем учебном году более двух оценок 4 и/или 5 баллов по результатам промежуточной аттестации до пересдач – по 10-балльной шкале; или в получении по результатам промежуточной аттестации (до пересдач) оценки ниже 4 баллов по десятибалльной шкале; или в наличии неявок на аттестационные испытания без уважительной с Порядком студент может претендовать на переход на бесплатное обучение (при наличии вакантного бюджетного места на образовательной программе) при соблюдении условий: На момент подачи заявления не имеет: академических задолженностей и не обучается в связи с этим по индивидуальному учебному плану специального типа с повторным изучением ряда дисциплин, дисциплинарных взысканий, задолженности по оплате обучения . 2\\. И соответствует одному из следующих условий: а) Сдача* экзаменов за последний семестр** обучения, предшествующий подаче заявления, на оценки "отлично" или "отлично" и "хорошо" или "хорошо"; б) Отнесение к следующему числу лиц: детей-сирот, оставшихся без попечения родителей, а также лицам из числа детей-сирот и детей, оставшихся без попечения родителей; граждан в возрасте до двадцати лет, имеющих только одного родителя — инвалида I группы, если среднедушевой доход семьи ниже величины прожиточного минимума, установленного в соответствующем субъекте Российской Федерации; женщин, родивших ребенка в период обучения; детей лиц, принимающих или принимавших участие в специальной военной операции на территориях Украины, Донецкой Народной Республики, Луганской Народной Республики, Запорожской области и Херсонской области (далее - «Аллегро» с их последующим списанием на премиальные (бесплатные) билеты; специальные предложения партнеров программы. Условия участия для студентов НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) - Санкт-Петербург Условия участия для студентов НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) - Нижний Новгород Условия участия для студентов НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) - Пермь Для участия в программе необходимо: Самостоятельно зарегистрироваться на сайте программы «РЖД Бонус» Получить справку, подтверждающую факт обучения Отправить справку по форме обратной связи в личном кабинете. Скидка будет присвоена в течение 2-х суток с момента отправки справки. !!! Упрощенная схема получения скидки действует теперь для всех студентов и аспирантов! Студенты старше 23 лет могут теперь самостоятельно через личный кабинет на сайте Программы направлять справки. Скидка действует до 1 сентября следующего учебного года. Для продления скидки необходимо отправить справку, выданную в новом учебном году, или повторно обратиться в Управление социальной сферы. С подробной информацией о программе «РЖД Бонус» можно ознакомиться на сайте www.rzd-bonus.ru</t>
         </is>
       </c>
-      <c r="K17" t="n">
+      <c r="L17" t="n">
         <v>2</v>
       </c>
-      <c r="L17" t="n">
+      <c r="M17" t="n">
         <v>23</v>
       </c>
-      <c r="M17" t="n">
+      <c r="N17" t="n">
         <v>11.5</v>
       </c>
-      <c r="N17" t="n">
+      <c r="O17" t="n">
         <v>0.9130434782608695</v>
       </c>
-      <c r="O17" t="n">
+      <c r="P17" t="n">
         <v>0.858106255531311</v>
       </c>
-      <c r="P17" t="n">
+      <c r="Q17" t="n">
         <v>0.04120418429374695</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="R17" t="n">
         <v>0.1006895527243614</v>
       </c>
-      <c r="R17" t="n">
+      <c r="S17" t="n">
         <v>2.823707258448521</v>
       </c>
-      <c r="S17" t="n">
+      <c r="T17" t="n">
         <v>0.4735427498817444</v>
       </c>
-      <c r="T17" t="n">
+      <c r="U17" t="n">
         <v>0.5037152171134949</v>
       </c>
-      <c r="U17" t="n">
+      <c r="V17" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0.4984391927719116</v>
+      </c>
+      <c r="X17" t="n">
         <v>2.790522</v>
       </c>
     </row>
@@ -1885,44 +2076,55 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы?  Подробнее: https://nnov.hse.ru/aup/sdu/ https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>-1</v>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="n">
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="n">
         <v>4</v>
       </c>
-      <c r="L18" t="n">
+      <c r="M18" t="n">
         <v>22</v>
       </c>
-      <c r="M18" t="n">
+      <c r="N18" t="n">
         <v>5.5</v>
       </c>
-      <c r="N18" t="n">
+      <c r="O18" t="n">
         <v>0.9545454545454546</v>
       </c>
-      <c r="O18" t="n">
+      <c r="P18" t="n">
         <v>0.04583731293678284</v>
       </c>
-      <c r="P18" t="n">
+      <c r="Q18" t="n">
         <v>0.9369155764579773</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="R18" t="n">
         <v>0.01724718324840069</v>
       </c>
-      <c r="R18" t="n">
+      <c r="S18" t="n">
         <v>0</v>
       </c>
-      <c r="S18" t="n">
+      <c r="T18" t="n">
         <v>0.08242271840572357</v>
       </c>
-      <c r="T18" t="n">
+      <c r="U18" t="n">
         <v>0.6400665044784546</v>
       </c>
-      <c r="U18" t="n">
+      <c r="V18" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0.6237279772758484</v>
+      </c>
+      <c r="X18" t="n">
         <v>2.902921</v>
       </c>
     </row>
@@ -1964,44 +2166,55 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы?  Подробнее: https://nnov.hse.ru/aup/sdu/ https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>1</v>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="n">
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="n">
         <v>4</v>
       </c>
-      <c r="L19" t="n">
+      <c r="M19" t="n">
         <v>22</v>
       </c>
-      <c r="M19" t="n">
+      <c r="N19" t="n">
         <v>5.5</v>
       </c>
-      <c r="N19" t="n">
+      <c r="O19" t="n">
         <v>0.9545454545454546</v>
       </c>
-      <c r="O19" t="n">
+      <c r="P19" t="n">
         <v>0.04583731293678284</v>
       </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
         <v>0.9369155764579773</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="R19" t="n">
         <v>0.01724718324840069</v>
       </c>
-      <c r="R19" t="n">
+      <c r="S19" t="n">
         <v>0</v>
       </c>
-      <c r="S19" t="n">
+      <c r="T19" t="n">
         <v>0.08242271840572357</v>
       </c>
-      <c r="T19" t="n">
+      <c r="U19" t="n">
         <v>0.6400665044784546</v>
       </c>
-      <c r="U19" t="n">
+      <c r="V19" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.6237279772758484</v>
+      </c>
+      <c r="X19" t="n">
         <v>3.10213</v>
       </c>
     </row>
@@ -2043,48 +2256,59 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Социальные вопросы', 'Другое', 'Деньги', 'Другое', 'Учебный процесс', 'ГИА', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Социальные вопросы', 'ОВЗ', 'Выпускникам', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Социальные вопросы', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
           <t>Место за счет ВШЭ (Высшая школа экономики) - это бюджетное место, финансируемое непосредственно университетом. Претендовать на перевод на такое место могут студенты, успешно осваивающие образовательную программу и соответствующие определенным критериям, например, являющиеся участниками СВО или детьми участников СВО. Для перевода необходимо написать заявление и отправить его на электронный адрес perevod@hse.ru со своего корпоративного адреса.  Подробнее: https://www.hse.ru/scholarships/name\_mon https://www.hse.ru/studyspravka/rate https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>-1</v>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>ных братьев и сестер. Обучение за счет собственных средств Вышки будет доступно в том числе тем, кто уже учится в Вышке на коммерческой основе. Единственным условием для перевода с платных мест на обучение за счет средств университета является успешное освоение образовательной программы (без неудовлетворительных оценок по итогам последних сессий). Критерии перехода на бюджетные места / места за счет средств НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Студент может претендовать на перевод на бюджетное место / место за счет средств НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) при соблюдении следующих условий: является участником СВО / ребенком или близким родственником (супруги / родные братья и сестры) участника СВО; успешно освавает образовательную программу (без неудовлетворительных оценок по итогам последних сессий). Процедура перевода Подготовьте электронное письмо-заявление Электронное письмо должно быть направлено на почту perevod@hse.ru со своего корпоративного электронного адреса с темой «Перевод на место за счет НИУ (Национальный исследовательский университет) ВШЭ». В письме должна быть указана информация о Вас: ФИО Дата время обучения в НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) За что назначается (критерии отбора) За высокие научные (литературные, исследовательские) достижения во время обучения в НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Когда назначается В октябре публикуется приказ Минобрнауки России по утверждению стипендиатов На какой период времени назначается На 1 учебный год (сентябрь - август) Процедура подачи заявки на конкурс/порядок назначения стипендии без конкурса Заявки подаются в электронном виде в феврале-марте. К заявке прикрепляются документы, подтверждающие научные и учебные достижения участника конкурса. Отбор кандидатов от НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) проводит ученый совет НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики). Стипендиатов утверждает комиссия Минобрнауки России. Основания досрочного прекращения выплаты стипендии Отчисление из вуза, наличие оценок «удовлетворительно» и академической задолженности</t>
         </is>
       </c>
-      <c r="K20" t="n">
+      <c r="L20" t="n">
         <v>5</v>
       </c>
-      <c r="L20" t="n">
+      <c r="M20" t="n">
         <v>56</v>
       </c>
-      <c r="M20" t="n">
+      <c r="N20" t="n">
         <v>11.2</v>
       </c>
-      <c r="N20" t="n">
+      <c r="O20" t="n">
         <v>0.8928571428571429</v>
       </c>
-      <c r="O20" t="n">
+      <c r="P20" t="n">
         <v>0.9111878871917725</v>
       </c>
-      <c r="P20" t="n">
+      <c r="Q20" t="n">
         <v>0.03874489665031433</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="R20" t="n">
         <v>0.05006717890501022</v>
       </c>
-      <c r="R20" t="n">
+      <c r="S20" t="n">
         <v>18.83879720134051</v>
       </c>
-      <c r="S20" t="n">
+      <c r="T20" t="n">
         <v>0.6349400281906128</v>
       </c>
-      <c r="T20" t="n">
+      <c r="U20" t="n">
         <v>0.4750597476959229</v>
       </c>
-      <c r="U20" t="n">
+      <c r="V20" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0.2951933741569519</v>
+      </c>
+      <c r="X20" t="n">
         <v>4.031493</v>
       </c>
     </row>
@@ -2126,48 +2350,59 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
+          <t>['Наука', 'Другое', 'Наука', 'Другое', 'Наука', 'Другое', 'Наука', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
           <t>Чтобы провести научное исследование, Вы можете обратиться к ресурсам Высшей школы экономики. ВШЭ предлагает различные проекты и программы поддержки научных инициатив, такие как Школа научного вики-редактора, где студенты могут приобрести навыки научной редактуры в Википедии. Кроме того, в ВШЭ функционируют научные лаборатории и центры, занимающиеся различными направлениями исследований. Например, Институт демографии имени А.Г. Вишневского, Центр исследований гражданского общества и некоммерческого сектора, Центр трудовых исследований и другие. Для получения дополнительной информации и поддержки в проведении исследования, Вы можете обратиться в соответствующие подразделения ВШЭ или принять участие в одной из предлагаемых программ.  Подробнее: https://www.hse.ru/evaluation/instructors\_techfaq https://www.hse.ru/evaluation/instructors\_access https://studscience.hse.ru/snoscience https://www.hse.ru/scholarships/name\_mon</t>
         </is>
       </c>
-      <c r="I21" t="n">
+      <c r="J21" t="n">
         <v>1</v>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>ды СНО. Подать заявку на вступление в СНО НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Проекты Республика ученых Scientarium: школа молодых ученых Научные бои Научные кураторы Научная инициатива Конкурс научно-исследовательских работ студентов Поддержка участия в научных мероприятиях. Travel-grant Поддержка и проведение научных мероприятий Фестивали науки Собака@Павлова Zoomer Фестиваль науки "5 шагов" Фестиваль науки НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) «Наука³» Ярмарка лабораторий Документы СНО НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Положение о СНО НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Наши партнёры Научный комитет Студенческого совета НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Наши соц. сети</t>
         </is>
       </c>
-      <c r="K21" t="n">
+      <c r="L21" t="n">
         <v>8</v>
       </c>
-      <c r="L21" t="n">
+      <c r="M21" t="n">
         <v>93</v>
       </c>
-      <c r="M21" t="n">
+      <c r="N21" t="n">
         <v>11.625</v>
       </c>
-      <c r="N21" t="n">
+      <c r="O21" t="n">
         <v>0.8172043010752689</v>
       </c>
-      <c r="O21" t="n">
+      <c r="P21" t="n">
         <v>0.9133557677268982</v>
       </c>
-      <c r="P21" t="n">
+      <c r="Q21" t="n">
         <v>0.07078995555639267</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="R21" t="n">
         <v>0.01585431396961212</v>
       </c>
-      <c r="R21" t="n">
+      <c r="S21" t="n">
         <v>21.52611805045797</v>
       </c>
-      <c r="S21" t="n">
+      <c r="T21" t="n">
         <v>0.5431994795799255</v>
       </c>
-      <c r="T21" t="n">
+      <c r="U21" t="n">
         <v>0.409995824098587</v>
       </c>
-      <c r="U21" t="n">
+      <c r="V21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="W21" t="n">
+        <v>0.1722756326198578</v>
+      </c>
+      <c r="X21" t="n">
         <v>4.587115</v>
       </c>
     </row>
@@ -2209,48 +2444,59 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
+          <t>['Наука', 'Другое', 'Наука', 'Другое', 'Наука', 'Другое', 'Наука', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
           <t>В НИУ ВШЭ существует множество возможностей для развития в науке. Университет предлагает различные лаборатории и центры, такие как Форсайт-центр, Лаборатория исследований науки и технологий, Лаборатория молекулярной физиологии и другие. Также есть портал Академического развития, который предоставляет доступ к образовательным ресурсам и инструментам академического развития. Кроме того, в НИУ ВШЭ проводятся различные мероприятия, такие как дни центров, семинары и конференции. Для студентов и сотрудников доступны подкасты, где обсуждаются актуальные исследования и пути в науке.  Подробнее: https://www.hse.ru/org/units/general\_activity/218401398/ http://academics.hse.ru/ https://www.hse.ru/science/facilities https://www.hse.ru/science/social#pagetop</t>
         </is>
       </c>
-      <c r="I22" t="n">
+      <c r="J22" t="n">
         <v>1</v>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>стественные науки Медицинские науки Биология Здравоохранение Телефон: +7 (495) 772-95-90 , доб. 11756 Email: omaximova@hse.ru Москва, Мясницкая ул., д. 11 Институт статистических исследований и экономики знаний → Форсайт-центр Лаборатория исследований науки и технологий Социальные науки Экономика и менеджмент Москва, Профсоюзная ул., 33, к.4 Учебные подразделения → Факультет биологии и биотехнологии Лаборатория молекулярной физиологии Естественные науки Биология Email: ekoltsova@hse.ru Санкт-Петербург, Седова ул., 55 корп. 2, лит. А НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) в Санкт-Петербурге → Санкт-Петербургская школа социальных наук Лаборатория социальной и когнитивной информатики Естественные науки Социальные науки Гуманитарные науки Математика Психология Социология (включая демографию и антропологию) Филология и лингвистика Телефон: +7 (495) 772-95-90 , доб. 12244 Email: lcsr.event@hse.ru Москва, Мясницкая ул., д. 20 +7 (495) 772-Управление академического развития Портал Академического развития предназначен для содействия профессиональному росту преподавателей, научных сотрудников и аспирантов. Портал обеспечивает доступ к современным образовательным ресурсам и ключевым инструментам академического развития Вышки, а также способствует созданию единого безбарьерного информационного пространства. Новости Что нового в библиотеке ИИ-ресурсов? 17 октября, 2024 г. идеи и опыт Центр академического письма День Центра 2024: что нового мы узнали? 2 октября, 2024 г. Образование репортаж о событии Центр академического письма ИИ: угроза или возможность? 20 сентября, 2024 г. Экспертиза Центр академического письма Highlights of the academic year 2023-2024 2 сентября, 2024 г. Образование Центр академического письма Пополнение в библиотеке Центра академического письма 9 июля, 2024 г. Экспертиза Центр академического письма Первые результаты реализации Инициативных академических проектов 2023 5 июля, 2024 г. идеи и опыт репортаж о событии Академический кадровый резерв НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Все новости ; уникальная научная установка «Автоматизированная система неинвазивной стимуляции мозга с возможностью синхронной регистрации биотоков мозга и отслеживанию фиксации глазодвижения» ; Программная система для поиска информации и обнаружения знаний из различных источников данных на основе подхода FCA ; многофункциональный инновационный телевизионный технический центр ; видеостудия OneButton ; Bloomberg professional, Bureau van Dijk (Ruslana, Zephir, Amadeus), Capital IQ, COMPUSTAT (Global) и другие базы данных Школы финансов факультета экономических наук; доступ к материально- технической базе ведущих физических институтов РАН: Института космических исследований , Института физики твердого тела , Института физических проблем им. П.Л. Капицы , Института спектроскопии , Института общей физики им. А.М. Прохорова , Институт теоретической физики им. Л.Д. Ландау ; уникальное оборудование для когнитивных исследований и исследований в области нейроэкономики ; «клетка Фарадея» — многослойная комната, защищенная от помех и излучений; подписка на десятки баз зарубежной и отечественной периодики ; комплексная система социологических обследований «Мониторинг экономики образования» , которую НИ</t>
         </is>
       </c>
-      <c r="K22" t="n">
+      <c r="L22" t="n">
         <v>6</v>
       </c>
-      <c r="L22" t="n">
+      <c r="M22" t="n">
         <v>75</v>
       </c>
-      <c r="M22" t="n">
+      <c r="N22" t="n">
         <v>12.5</v>
       </c>
-      <c r="N22" t="n">
+      <c r="O22" t="n">
         <v>0.7333333333333333</v>
       </c>
-      <c r="O22" t="n">
+      <c r="P22" t="n">
         <v>0.8897854685783386</v>
       </c>
-      <c r="P22" t="n">
+      <c r="Q22" t="n">
         <v>0.05692800879478455</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="R22" t="n">
         <v>0.05328654125332832</v>
       </c>
-      <c r="R22" t="n">
+      <c r="S22" t="n">
         <v>17.57755485657643</v>
       </c>
-      <c r="S22" t="n">
+      <c r="T22" t="n">
         <v>0.6261861324310303</v>
       </c>
-      <c r="T22" t="n">
+      <c r="U22" t="n">
         <v>0.5444013476371765</v>
       </c>
-      <c r="U22" t="n">
+      <c r="V22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0.2031240016222</v>
+      </c>
+      <c r="X22" t="n">
         <v>3.903575</v>
       </c>
     </row>
@@ -2292,44 +2538,55 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Другое', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Другое', 'Учебный процесс', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
           <t>Вас могут отчислить из НИУ ВШЭ за не выполнение обязанностей по добросовестному освоению образовательной программы и выполнению учебного плана. Это может произойти, например, если вы не явились на государственное аттестационное испытание по уважительной причине и не представили заключение врачебной комиссии о необходимости предоставления академического отпуска по медицинским показаниям. Также отчисление может быть применено как мера дисциплинарного взыскания за нарушение академических норм, включая плагиат в ВКР.  Подробнее: https://www.hse.ru/studyspravka/Skidki https://nnov.hse.ru/aup/sdu/ https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I23" t="n">
+      <c r="J23" t="n">
         <v>1</v>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="n">
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="n">
         <v>4</v>
       </c>
-      <c r="L23" t="n">
+      <c r="M23" t="n">
         <v>66</v>
       </c>
-      <c r="M23" t="n">
+      <c r="N23" t="n">
         <v>16.5</v>
       </c>
-      <c r="N23" t="n">
+      <c r="O23" t="n">
         <v>0.8939393939393939</v>
       </c>
-      <c r="O23" t="n">
+      <c r="P23" t="n">
         <v>0.0405488945543766</v>
       </c>
-      <c r="P23" t="n">
+      <c r="Q23" t="n">
         <v>0.9503394365310669</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="R23" t="n">
         <v>0.009111762978136539</v>
       </c>
-      <c r="R23" t="n">
+      <c r="S23" t="n">
         <v>0</v>
       </c>
-      <c r="S23" t="n">
+      <c r="T23" t="n">
         <v>0.05277250334620476</v>
       </c>
-      <c r="T23" t="n">
+      <c r="U23" t="n">
         <v>0.3621701002120972</v>
       </c>
-      <c r="U23" t="n">
+      <c r="V23" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="W23" t="n">
+        <v>0.394547164440155</v>
+      </c>
+      <c r="X23" t="n">
         <v>4.253274</v>
       </c>
     </row>
@@ -2371,48 +2628,59 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Учебный процесс', 'Выпускникам', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Наука', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы?  Подробнее: https://www.hse.ru/studyspravka/wes https://www.hse.ru/evaluation/#timetable https://www.hse.ru/scholarships/social\_scholarship\_new https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I24" t="n">
+      <c r="J24" t="n">
         <v>-1</v>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>языке можно не переводить (оставить на языке оригинала), но желательно перевести название города/штата/провинции/страны. Нашли опечатку ? Выделите её, нажмите Ctrl+Enter и отправьте нам уведомление. Спасибо за участие! Сервис предназначен только для отправки сообщений об орфографических и пунктуационных ошибках. Отправка бумажных копий документов в WES Если Вам требуется отправить бумажные копии документов в WES, закажите заверенные копии документов в электронном сервисе Центра сервиса «Студент» по ссылке https://pmo.hse.ru/servicedesk/customer/portal/93/group/221 . Важно: для подачи заявки необходимо авторизоваться в Едином личном кабинете. Если у Вас нет аккаунта в ЕЛК (единый личный кабинет), пожалуйста, зарегистрируйтесь по ссылке . Получите уведомление о готовности документов и посетите Центр сервиса «Студент» (при себе необходимо иметь паспорт). Сотрудник Центра сервиса «Студент» запечатает документ(ы) в конверт, проставит фирменный штамп НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) и передаст Вам конверт для самостоятельной отправки документов в адрес WES. Остались вопросы? Напишите нам на почту studcentre@hse.ru– Медицинское освидетельствование Приказ Министерства здравоохранения РФ №1079Н По договору НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) с "Городской поликлиникой №3 ДЗМ" медицинское освидетельствование высоко-квалифицированных специалистов (ВКС) проводится за счет НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики). На основании приказа Министерства здравоохранения РФ №1079Н иностранные граждане обязаны проходить обязательное медицинское освидетельствование, включающее: лабораторные исследования на наличие инфекционных заболеваний химико-токсикологические исследования на наличие в организме наркотических и психотропных веществ исследование крови флюорография/рентгенография иммунодиагностика бактериоскопические исследования и др. Иностранный гражданин должен иметь при себе: документ удостоверяющий личность (оригинал и копия), перевод паспорта (копия), миграционная карта (оригинал и копия), учебная виза для студентов (копия), разрешение на работу для преподавателей, ВКС,КС, квота (оригинал и копия), регистрация (копия). Важно! Для выполнения достоверных лабораторных исследований не употреблять пищу до медицинского</t>
         </is>
       </c>
-      <c r="K24" t="n">
+      <c r="L24" t="n">
         <v>4</v>
       </c>
-      <c r="L24" t="n">
+      <c r="M24" t="n">
         <v>22</v>
       </c>
-      <c r="M24" t="n">
+      <c r="N24" t="n">
         <v>5.5</v>
       </c>
-      <c r="N24" t="n">
+      <c r="O24" t="n">
         <v>0.9545454545454546</v>
       </c>
-      <c r="O24" t="n">
+      <c r="P24" t="n">
         <v>0.8077396154403687</v>
       </c>
-      <c r="P24" t="n">
+      <c r="Q24" t="n">
         <v>0.08586805313825607</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="R24" t="n">
         <v>0.1063923016190529</v>
       </c>
-      <c r="R24" t="n">
+      <c r="S24" t="n">
         <v>5.583218697652022</v>
       </c>
-      <c r="S24" t="n">
+      <c r="T24" t="n">
         <v>0.5180344581604004</v>
       </c>
-      <c r="T24" t="n">
+      <c r="U24" t="n">
         <v>0.4906268119812012</v>
       </c>
-      <c r="U24" t="n">
+      <c r="V24" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="W24" t="n">
+        <v>0.4755246639251709</v>
+      </c>
+      <c r="X24" t="n">
         <v>3.150178</v>
       </c>
     </row>
@@ -2454,48 +2722,59 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Деньги', 'Учебный процесс', 'Цифровые системы', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Наука', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
           <t>Ваш рейтинг в SmartLMS можно узнать в разделе "Оцени свои курсы" после входа в личный кабинет. Вы также можете проверить свой рейтинг на сайте вашей образовательной программы в разделе "Студентам - Рейтинги". Помните, что рейтинг может влиять на различные аспекты вашего обучения, включая получение скидок на оплату обучения, выбор популярных дисциплин и возможность получения грантов на академическую международную мобильность.  Подробнее: https://www.hse.ru/evaluation/students\_techguide https://www.hse.ru/evaluation/instructors\_access https://www.hse.ru/studyspravka/rate https://www.hse.ru/studyspravka/step</t>
         </is>
       </c>
-      <c r="I25" t="n">
+      <c r="J25" t="n">
         <v>-1</v>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>Техническая инструкция_ Техническая инструкция Поиск и открытие анкеты Технические проблемы в структуре анкеты Технические особенности заполнения анкеты. Анонимность Нестандартные вопросы Поиск и открытие анкеты Когда проходит оценка? Форма для оценки преподавателей и дисциплин открывается в личном кабинете студента в LMS (Learning management system) за три недели до начала сессии. График проведения СОП (студенческая оценка преподавания) можно посмотреть по ссылке . Как открыть анкету? Анкета СОП (студенческая оценка преподавания) доступна в LMS (Learning management system). Чтобы зайти в личный кабинет в LMS (Learning management system), необходимо перейти по ссылке и ввести свои логин и пароль от Единого личного кабинета. Если у вас есть проблемы со входом — читайте инструкцию. На главной странице LMS (Learning management system) после ввода логина и пароля перейдите в модуль с анкетами по кнопке «Оцени свои курсы». Для открытия модуля с анкетами вы также можете воспользоваться прямой ссылкой «Пройти СОП» вверху страницы. Далее в самом модуле необходимо выбрать текущий учебный период и заполнить анкету. Местонахождение модуля «Оцени свои курсы» в LMS (Learning management system) С сайтаЭлектронное портфолио студента Электронное портфолио студента НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) В НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) на базе on-line системы обучения Learning Management System (LMS (Learning management system)) разработан сервис «Электронное портфолио студента (СтЭП)», который доступен в LMS (Learning management system) после предварительной авторизации и разработан на русском и английском языках. СтЭП позволяет зафиксировать достижения студентов по следующим видам деятельности: учебная; научная; практики и проектная; культурно-творческая; общественная; спортивная; дополнительное образование. В рамках учебной деятельности бóльшая часть информации автоматически интегрируется в портфолио студента из учетной системы НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики): информация об успеваемости студента, выполненные курсовые и выпускные квалификационные работы, исходящая мобильность внутри страны или на международном уровне с указанием изученных дисциплин. Здесь же дополнительно производится расчет текущего показателя GPA (Grade Point Average), на основании которого определяется успеваемость студента во многих зарубежных университетах. Для студентов, имеющих публикации в науч, в открытом доступе на сайтах образовательных программ в разделе Студентам - Рейтинги. На что влияет место в рейтинге Рейтинговая позиция часто используется для распределения различных студенческих благ. Студентам, которые оплачивают свое обучение, хорошее место в рейтинге может принести скидку на оплату обучения . Место в рейтинге может повлиять на возможность записаться на популярные дисциплины по выбору, майноры, общеуниверситетские факультативы . При принятии решения о выделении студенту гранта на академическую международную мобильность , также важную роль может сыграть ваш рейтинг. Как рассчитывается рейтинг Рейтинг определяется следующим образом: Каждый факультет принимает решение какие студенты будут друг с другом сравниваться. Возможно сравнение студентов одного курса одной образовательной программы, либо нескольких образовательных программ Для каждого студента определяется сумма произведений оценок на кредитный вес элемента учебного плана. Например, студент в течение полугодия изучал английский язык (4 кредита), математический анализ (5 кредитов) и историю (3 кредита). Получил по ним такие оценки: 8, 7, 10. Для этого студента рассчитывается показатель: 4*8+5*7+3*10 = 97. Так как у каждого студента Вышки учебный план индивидуальный, то, чем старше курс, тем разнообразнее набор</t>
         </is>
       </c>
-      <c r="K25" t="n">
+      <c r="L25" t="n">
         <v>4</v>
       </c>
-      <c r="L25" t="n">
+      <c r="M25" t="n">
         <v>59</v>
       </c>
-      <c r="M25" t="n">
+      <c r="N25" t="n">
         <v>14.75</v>
       </c>
-      <c r="N25" t="n">
+      <c r="O25" t="n">
         <v>0.8305084745762712</v>
       </c>
-      <c r="O25" t="n">
+      <c r="P25" t="n">
         <v>0.9635700583457947</v>
       </c>
-      <c r="P25" t="n">
+      <c r="Q25" t="n">
         <v>0.01216941513121128</v>
       </c>
-      <c r="Q25" t="n">
+      <c r="R25" t="n">
         <v>0.02426047623157501</v>
       </c>
-      <c r="R25" t="n">
+      <c r="S25" t="n">
         <v>12.55593099685346</v>
       </c>
-      <c r="S25" t="n">
+      <c r="T25" t="n">
         <v>0.6039144992828369</v>
       </c>
-      <c r="T25" t="n">
+      <c r="U25" t="n">
         <v>0.5474289059638977</v>
       </c>
-      <c r="U25" t="n">
+      <c r="V25" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.3907949328422546</v>
+      </c>
+      <c r="X25" t="n">
         <v>3.718311</v>
       </c>
     </row>
@@ -2537,48 +2816,59 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
           <t>Чтобы перевестись с коммерческого места на бюджетное, необходимо обратиться к специалистам по сопровождению отдельных категорий студентов. Они проверят наличие оснований для перевода. Если на образовательной программе имеются вакантные бюджетные места, возможно предложение о переводе на бюджетное место или место за счет средств НИУ ВШЭ. После рассмотрения документов будет издан приказ о вашем переходе на бюджетное место. Перевод осуществляется с даты отправки письма-заявления. Важно отметить, что перевод на бюджетное место возможен при отсутствии академических задолженностей и активном обучении. Для оформления заявки на перевод на бесплатное обучение можно воспользоваться модулем "Заявка на ВБМ" в личном кабинете в системе LMS НИУ ВШЭ. Решение о переходе на бюджетное место принимается общеуниверситетской комиссией с учетом мнения Студенческого совета НИУ ВШЭ.  Подробнее: https://www.hse.ru/studyspravka/programme\_change https://www.hse.ru/studyspravka/perbud</t>
         </is>
       </c>
-      <c r="I26" t="n">
+      <c r="J26" t="n">
         <v>-1</v>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>Перевод на бесплатное обучение Перевод с платного обучения на бесплатное Перевод по общим основаниям Основная информация Протоколы общеуниверситетской комиссии Регламентирующие документы Перевод по льготным основаниям (участники СВО, их дети и близкие родственники) Основная информация Критерии перевода Процедура перевода Перевод на бесплатное обучение по общим основаниям Основные критерии перехода на бюджет Порядок и критерии перевода студента с платного обучения на бесплатное установлены приказом Минобрнауки РФ от 28.08.2023 № 822 " Об утверждении порядка и случаев перехода лиц, обучающихся по образовательным программам среднего профессионального и высшего образования, с платного обучения на обучение за счет средств бюджетных ассигнований федерального бюджета, бюджетов субъектов Российской Федерации и местных бюджетов либо за счет собственных средств организации, осуществляющей образовательную деятельность, в том числе средств, полученных от приносящей доход деятельности, добровольных пожертвований и целевых взносов физических и (или) юридических лиц " В соответствии с Порядком студент может претендовать на переход на бесплатное обучение (при наличии вакантного бюджетного места на образовательной программе) при соблюдении условий: На момент подачи заявления не имеет: академических задолженностей и не обучается таких переводов не предусмотрены, поэтому заявления рассматриваются в любое время (в отличие от перевода с одной ОП на другую с отчислением). Перевод на другую программу студента, обучающегося в пределах квоты Правительства РФ Основная информация Перевод иностранного студента, обучающегося на бюджетной основе в пределах квоты Правительства РФ возможен в рамках одной укрупненной группы направлений/специальностей* (с изменением направления подготовки / без изменения). В случае изменения направления подготовки (в рамках одной укрупненной группы) перевод возможен только при наличии письменного согласия Министерства науки и высшего образования РФ. Перевод на полностью платные образовательные программы возможен только на вакантное коммерческое место (при их наличии). * Укрупненная группа - группа, в состав которой входят направления подготовки, по которым реализуются образовательные программы. Например, если Вы обучаетесь по образовательной программе «Экономика» направления подготовки 38.03.01 Экономика, то перевод возможен на образовательные программы, которые реализуются по направлениям подготовки, начинающимся с 38.00.00 (перевод на образовательную программу «Дизайн» по направлению подготовки 54.03.01 Дизайн невозможен). В случае если в направлении на обучение, выданном Минобрнауки России, указано, что Вы направлены на обучение</t>
         </is>
       </c>
-      <c r="K26" t="n">
+      <c r="L26" t="n">
         <v>9</v>
       </c>
-      <c r="L26" t="n">
+      <c r="M26" t="n">
         <v>117</v>
       </c>
-      <c r="M26" t="n">
+      <c r="N26" t="n">
         <v>13</v>
       </c>
-      <c r="N26" t="n">
+      <c r="O26" t="n">
         <v>0.7435897435897436</v>
       </c>
-      <c r="O26" t="n">
+      <c r="P26" t="n">
         <v>0.9350264072418213</v>
       </c>
-      <c r="P26" t="n">
+      <c r="Q26" t="n">
         <v>0.01945932954549789</v>
       </c>
-      <c r="Q26" t="n">
+      <c r="R26" t="n">
         <v>0.04551419988274574</v>
       </c>
-      <c r="R26" t="n">
+      <c r="S26" t="n">
         <v>23.46294018906321</v>
       </c>
-      <c r="S26" t="n">
+      <c r="T26" t="n">
         <v>0.6311159729957581</v>
       </c>
-      <c r="T26" t="n">
+      <c r="U26" t="n">
         <v>0.4619488120079041</v>
       </c>
-      <c r="U26" t="n">
+      <c r="V26" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.3907797336578369</v>
+      </c>
+      <c r="X26" t="n">
         <v>5.136272</v>
       </c>
     </row>
@@ -2620,48 +2910,59 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Траектории обучения', 'Социальные вопросы', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Дополнительное образование', 'Социальные вопросы', 'Общежития', 'Другое', 'Деньги', 'Социальные вопросы', 'Другое', 'Деньги', 'Другое', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Английский язык', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование']</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>В НИУ ВШЭ предусмотрены различные стипендии, включая стипендию "Серебряный птенец", которая присуждается за успешную учебу и научную деятельность. Размер этой стипендии составляет 10 000 рублей ежемесячно на протяжении всего периода обучения. Кроме того, существуют именные стипендии выдающихся ученых. Также стоит отметить программу лояльности "РЖД Бонус", предоставляющую студентам скидки на железнодорожные билеты.  Подробнее: https://spasibo.hse.ru/ https://www.hse.ru/scholarships/silver</t>
         </is>
       </c>
-      <c r="I27" t="n">
+      <c r="J27" t="n">
         <v>-1</v>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>Стипендия НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) «Серебряный птенец» Стипендия НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) «Серебряный птенец» Именные стипендии: Выдающихся ученых НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Минобрнауки России «Серебряный птенец» Стипендия «Серебряный птенец» была учреждена в 2012 году в рамках ежегодной церемонии «Золотая Вышка» . Размер стипендии составляет 10 000 рублей ежемесячно в течение всего времени обучения в Вышке. Кандидаты на получение стипендии выдвигаются преподавателями ВШЭ (Высшая школа экономики) за успешную учёбу и научную деятельность. Победители выбираются большинством голосов жюри «Золотая Вышка». Читай истории успеха и становись Серебряным птенцом! Положение о стипендии "Серебряный птенец" - в Положении о стипендиальном обеспечении обучающихся НИУ (Национальный исследовательский университет) ВПожертвования Высшая школа экономики стала для многих символом качественного образования, высоких стандартов исследовательской работы, лабораторией инновационных идей и проектов. Мы живём в соответствии с понятными всем ценностями и готовы следовать им при любых внешних обстоятельствах. Мы научились зарабатывать на рынке и разумно вкладывать средства так, чтобы обеспечить постоянный рост, в том числе за счёт привлечения лучших преподавателей и учёных, высокопрофессиональных менеджеров и вдохновляющих лидеров. Вышка – амбициозный университет, находящийся в постоянном развитии. Сейчас нашей глобальной целью является закрепление позиции флагмана российского образования и получение международного признания в приоритетных областях научного знания. Достижение такой высокой цели невозможно без доверия и поддержки со стороны широкого сообщества, его выпускников, друзей и партнёров. С вашим участием мы можем сделать больше!</t>
         </is>
       </c>
-      <c r="K27" t="n">
+      <c r="L27" t="n">
         <v>5</v>
       </c>
-      <c r="L27" t="n">
+      <c r="M27" t="n">
         <v>52</v>
       </c>
-      <c r="M27" t="n">
+      <c r="N27" t="n">
         <v>10.4</v>
       </c>
-      <c r="N27" t="n">
+      <c r="O27" t="n">
         <v>0.9423076923076923</v>
       </c>
-      <c r="O27" t="n">
+      <c r="P27" t="n">
         <v>0.7783530354499817</v>
       </c>
-      <c r="P27" t="n">
+      <c r="Q27" t="n">
         <v>0.2040984928607941</v>
       </c>
-      <c r="Q27" t="n">
+      <c r="R27" t="n">
         <v>0.01754840277135372</v>
       </c>
-      <c r="R27" t="n">
+      <c r="S27" t="n">
         <v>18.46092029429211</v>
       </c>
-      <c r="S27" t="n">
+      <c r="T27" t="n">
         <v>0.6272159814834595</v>
       </c>
-      <c r="T27" t="n">
+      <c r="U27" t="n">
         <v>0.350657194852829</v>
       </c>
-      <c r="U27" t="n">
+      <c r="V27" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.2599422931671143</v>
+      </c>
+      <c r="X27" t="n">
         <v>3.815742</v>
       </c>
     </row>
@@ -2703,48 +3004,59 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Другое', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
           <t>Да, изучение русского языка является обязательным для иностранных студентов, обучающихся в НИУ ВШЭ на программах, где преподавание ведется не на английском языке. Это необходимо для успешного освоения учебного материала и достижения уровня владения русским языком, требуемого для академической и профессиональной деятельности.  Подробнее: https://www.hse.ru/studyspravka/russian https://www.hse.ru/studyspravka/edmodel\_bachelor\_20</t>
         </is>
       </c>
-      <c r="I28" t="n">
+      <c r="J28" t="n">
         <v>1</v>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Русский язык как иностранный Русский язык как иностранный (РКИ (русский язык как иностранный)) Данный раздел актуален только для студентов, поступивших не ранее 2024 года . Изучение русского языка – неотъемлемая часть успешного обучения в НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики). Владение русским языком значительно улучшает ваши образовательные перспективы в России. Почему иностранному студенту важно учить русский язык? Развитие русскоязычной коммуникативной компетенции для достижения уровня, необходимого для успешной академической и профессиональной деятельности (от ТРКИ-II до от ТРКИ-III [1] ), является частью образовательного стандарта НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) , и обязательно для всех иностранных студентов, обучающихся на образовательных программах, реализуемых не на английском языке. Недостаточный уровень русского языка не позволит студенту успешно осваивать учебный материал — многие дисциплины преподаются на русском языке. Низкий уровень языковой подготовки приведет к невозможности полноценно освоить всю образовательную программу. [1] Тестирование по русскому языку как иностранному языку (ТРКИ) основано на единой сертификационной системе определения уровня владения практическим русским язы</t>
         </is>
       </c>
-      <c r="K28" t="n">
+      <c r="L28" t="n">
         <v>3</v>
       </c>
-      <c r="L28" t="n">
+      <c r="M28" t="n">
         <v>42</v>
       </c>
-      <c r="M28" t="n">
+      <c r="N28" t="n">
         <v>14</v>
       </c>
-      <c r="N28" t="n">
+      <c r="O28" t="n">
         <v>0.9047619047619048</v>
       </c>
-      <c r="O28" t="n">
+      <c r="P28" t="n">
         <v>0.8994303941726685</v>
       </c>
-      <c r="P28" t="n">
+      <c r="Q28" t="n">
         <v>0.09433358907699585</v>
       </c>
-      <c r="Q28" t="n">
+      <c r="R28" t="n">
         <v>0.006235925946384668</v>
       </c>
-      <c r="R28" t="n">
+      <c r="S28" t="n">
         <v>27.34416665035725</v>
       </c>
-      <c r="S28" t="n">
+      <c r="T28" t="n">
         <v>0.6679060459136963</v>
       </c>
-      <c r="T28" t="n">
+      <c r="U28" t="n">
         <v>0.4767716825008392</v>
       </c>
-      <c r="U28" t="n">
+      <c r="V28" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.3605345487594604</v>
+      </c>
+      <c r="X28" t="n">
         <v>3.741623</v>
       </c>
     </row>
@@ -2786,48 +3098,59 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Наука', 'Другое', 'Учебный процесс', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
           <t>При использовании искусственного интеллекта (ИИ) в своих работах, вы должны указать это в соответствующем разделе вашей работы. Вам необходимо описать цели применения, название конкретной модели, адрес ее сайта в интернете (либо описания иного источника модели) и способ ее применения. Это требование установлено для соблюдения академических норм и правил.  Подробнее: https://library.hse.ru/ticket https://www.hse.ru/studyspravka/plagiat https://www.hse.ru/evaluation/instructors\_techfaq https://library.hse.ru/tdnet\_help</t>
         </is>
       </c>
-      <c r="I29" t="n">
+      <c r="J29" t="n">
         <v>1</v>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>применения — соответствующие изменения в интерфейсах загрузки уже появились. Инструкция по загрузке работ в LMS (Learning management system) содержит описание того, как и где именно студент должен сообщить об использовании искусственного интеллекта. Система проверки работ на недопустимые заимствования с января 2024 года использует плагин для распознавания сгенерированных текстов. В иных видах учебных работ, при использовании генеративных моделей при написании работ, студент/ группа студентов обязан сопроводить задание специальным разделом «Описание применения генеративной модели» с описанием целей применения, названия конкретной модели, адреса ее сайта в интернете (либо описания иного источника модели), и способа ее применения. Преподаватель может поставить оценку “0” за работу, в которой он усматривает признаки применения ИИ без отдельного уведомления студента об этом в своей работе. Либо, если использование ИИ было явно запрещено преподавателем. Важно: Использование генеративных моделей без указания на это установленным образом является нарушением академических норм. Важно: В случае выявления несоответствия загруженного в систему LMS (Learning management system) студентом файла ВКР (выпускная квалификационная работа) представленному им на защиту тексту ВКР (выпускная квалификационная работа) к студенту применяется дисциплинарноеПомощь спроблемами_ Помощь с проблемами В данных замечены ошибки или неточности: чего-то не хватает или что-то лишнее Отправьте заявку с изложением проблемы по ссылке или письмом на rating@hse.ru . Нет доступа к результатам, а они нужны очень срочно Напишите менеджеру департамента, школы или кафедры, где вы работаете или где ранее преподавали (и к чему относятся те результаты, которые срочно нужны), и попросите прислать результаты СОП (студенческая оценка преподавания) выгрузкой в виде файла. Если от них нет ответа, напишите с аналогичной просьбой на rating@hse.ru , переслав переписку. Иная проблема с результатами Оставьте заявку по ссылке или напишите письмо на rating@hse.ru . а еще позволяет производить новые продукты, не используя ограниченные ресурсы, например, нефть. А еще — это часть «Третьей миссии» Вышки. «Третья миссия» НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) — это политика по влиянию на развитие общества и внешней среды. Университет берет на себя ответственность за вклад в развитие территорий своего присутствия — в том числе экологическое — а мы ему помогаем. «Ответственная Вышка» — тоже проект «Третьей миссии». Он помогает студентам стать более экологичными, рассказывая об эко-проектах студентов и возможностях участия в них. Мы — не исключение. Ваш цифровой читательский, дедлайны возврата книг, адреса и время работы библиотек — всё это в одном приложении HSE App X. Скачать бесплатно Как это работает? Откройте цифровой читательский Покажите штрих-код сотруднику библиотеки Чтобы взять книгу, не нужно доставать пластиковый читательский или вспоминать его номер — просто поднесите смартфон к сканеру сотрудника библиотеки. Как добавить читательский в Apple Wallet и Google Pay? Откройте читательский Зайдите в раздел «Библиотека» в приложении Добавьте карту iOS: Нажмите на кнопку «Добав</t>
         </is>
       </c>
-      <c r="K29" t="n">
+      <c r="L29" t="n">
         <v>4</v>
       </c>
-      <c r="L29" t="n">
+      <c r="M29" t="n">
         <v>49</v>
       </c>
-      <c r="M29" t="n">
+      <c r="N29" t="n">
         <v>12.25</v>
       </c>
-      <c r="N29" t="n">
+      <c r="O29" t="n">
         <v>0.8571428571428571</v>
       </c>
-      <c r="O29" t="n">
+      <c r="P29" t="n">
         <v>0.9430363178253174</v>
       </c>
-      <c r="P29" t="n">
+      <c r="Q29" t="n">
         <v>0.02837743051350117</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="R29" t="n">
         <v>0.02858622744679451</v>
       </c>
-      <c r="R29" t="n">
+      <c r="S29" t="n">
         <v>14.05645609867222</v>
       </c>
-      <c r="S29" t="n">
+      <c r="T29" t="n">
         <v>0.5993086695671082</v>
       </c>
-      <c r="T29" t="n">
+      <c r="U29" t="n">
         <v>0.5162511467933655</v>
       </c>
-      <c r="U29" t="n">
+      <c r="V29" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0.3928089737892151</v>
+      </c>
+      <c r="X29" t="n">
         <v>3.722226</v>
       </c>
     </row>
@@ -2869,48 +3192,59 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Другое', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Другое', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Другое', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Наука', 'Другое']</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
           <t>Для подключения к LMS (Learning management system) НИУ ВШЭ, вам необходимо зайти на сайт https://lms.hse.ru/ и ввести свои учетные данные - логин и пароль от вашей корпоративной почты. Если у вас возникают проблемы с доступом, проверьте правильность введенных данных или обратитесь за помощью по указанным ссылкам в соответствующем разделе.  Подробнее: https://www.hse.ru/studyspravka/programme\_change</t>
         </is>
       </c>
-      <c r="I30" t="n">
+      <c r="J30" t="n">
         <v>0</v>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>НП(с) Каталог программ бакалавриата здесь . Каталог программ магистратуры здесь . Заполните заявку на перевод в LMS (Learning management system) Заявку необходимо подать через свой личный кабинет в LMS (Learning management system). Получите информационное письмо с бланком заявления В случае положительного результата технической экспертизы заявки на корпоративную электронную почту, использованную при входе в LMS (Learning management system), будет направлен бланк заявления с информацией о дальнейших шагах. Подпишите и направьте заявление менеджерам образовательных программ (принимающей и отпускающей) и своему академическому руководителю Со своей корпоративной электронной почты необходимо направить письмо со сканом заявления академическому руководителю и менеджеру своей образовательной программы, чтобы получить решение академического руководителя о переводе на другую программу. В копию письма необходимо в обязательном порядке поставить менеджера интересующей образовательной программы. Пройдите аттестационные испытания (при их наличии) Дождитесь решения образовательной программы о переводе Если аттестационная комиссия приняла положительное решение о переводе, сообщите менеджеру интересующей программы о принятом решении или отмените свое заявление. В случае положительного решения аттестационная комиссия определит: список элементов учебного плана, которые могут быть перезачтены; список дисциплин, подлежащих изучению или переат</t>
         </is>
       </c>
-      <c r="K30" t="n">
+      <c r="L30" t="n">
         <v>3</v>
       </c>
-      <c r="L30" t="n">
+      <c r="M30" t="n">
         <v>48</v>
       </c>
-      <c r="M30" t="n">
+      <c r="N30" t="n">
         <v>16</v>
       </c>
-      <c r="N30" t="n">
+      <c r="O30" t="n">
         <v>0.9791666666666666</v>
       </c>
-      <c r="O30" t="n">
+      <c r="P30" t="n">
         <v>0.8670245409011841</v>
       </c>
-      <c r="P30" t="n">
+      <c r="Q30" t="n">
         <v>0.0983620285987854</v>
       </c>
-      <c r="Q30" t="n">
+      <c r="R30" t="n">
         <v>0.03461344912648201</v>
       </c>
-      <c r="R30" t="n">
+      <c r="S30" t="n">
         <v>14.70397257342613</v>
       </c>
-      <c r="S30" t="n">
+      <c r="T30" t="n">
         <v>0.5662901997566223</v>
       </c>
-      <c r="T30" t="n">
+      <c r="U30" t="n">
         <v>0.3835065960884094</v>
       </c>
-      <c r="U30" t="n">
+      <c r="V30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0.3130568265914917</v>
+      </c>
+      <c r="X30" t="n">
         <v>4.045079</v>
       </c>
     </row>
@@ -2952,44 +3286,55 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
+          <t>['Деньги', 'Траектории обучения', 'Деньги', 'Учебный процесс', 'Социальные вопросы', 'Деньги', 'Учебный процесс', 'Социальные вопросы', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'ОВЗ']</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
           <t>Чтобы получать стипендию, студенту необходимо выполнить ряд условий. Во-первых, соответствовать критериям отбора, установленным для конкретного вида стипендии. Во-вторых, подать заявку в установленные сроки и в соответствии с инструкциями Центра международной студенческой мобильности и образовательных проектов. После подачи заявки и успешного участия в конкурсе, студент должен подтвердить факт своего участия в программе мобильности, предоставив необходимые документы в Центр. Выплата стипендии начинается после издания соответствующего приказа. Для некоторых видов стипендий требуется предоставление дополнительных документов, таких как мотивационное письмо, сертификаты, благодарности и другие доказательства внеучебной активности.  Подробнее: https://spb.hse.ru/socq/socscholarship https://www.hse.ru/scholarships/need https://www.hse.ru/studyspravka/benefits</t>
         </is>
       </c>
-      <c r="I31" t="n">
+      <c r="J31" t="n">
         <v>0</v>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="n">
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="n">
         <v>7</v>
       </c>
-      <c r="L31" t="n">
+      <c r="M31" t="n">
         <v>86</v>
       </c>
-      <c r="M31" t="n">
+      <c r="N31" t="n">
         <v>12.28571428571429</v>
       </c>
-      <c r="N31" t="n">
+      <c r="O31" t="n">
         <v>0.8488372093023255</v>
       </c>
-      <c r="O31" t="n">
+      <c r="P31" t="n">
         <v>0.9270554780960083</v>
       </c>
-      <c r="P31" t="n">
+      <c r="Q31" t="n">
         <v>0.06276696920394897</v>
       </c>
-      <c r="Q31" t="n">
+      <c r="R31" t="n">
         <v>0.01017749030143023</v>
       </c>
-      <c r="R31" t="n">
+      <c r="S31" t="n">
         <v>0</v>
       </c>
-      <c r="S31" t="n">
+      <c r="T31" t="n">
         <v>0.05592939630150795</v>
       </c>
-      <c r="T31" t="n">
+      <c r="U31" t="n">
         <v>0.3332600295543671</v>
       </c>
-      <c r="U31" t="n">
+      <c r="V31" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.2151342928409576</v>
+      </c>
+      <c r="X31" t="n">
         <v>4.653668</v>
       </c>
     </row>
@@ -3031,48 +3376,59 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Наука', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Учебный процесс']</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
           <t>Я могу ответить на ваш вопрос частично. Для изменения темы дипломной работы необходимо написать личное заявление на имя руководителя факультета с кратким обоснованием вашей просьбы. Заявление должно быть подано в учебный офис не позднее, чем за один календарный месяц до установленного срока представления итогового варианта курсовой работы. Чтобы узнать конкретные сроки и процедуры, рекомендуется обратиться в учебный офис вашей программы или факультет.  Подробнее: https://www.hse.ru/studyspravka/kursovrab https://pay.hse.ru/ https://www.hse.ru/studyspravka/perezach https://www.hse.ru/studyspravka/vkr</t>
         </is>
       </c>
-      <c r="I32" t="n">
+      <c r="J32" t="n">
         <v>0</v>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>разделение. Необходимо предложить тему курсовой работы, предлагаемого руководителя и обоснование выбора в модуле "Темы КР/ВКР" в системе LMS (Learning management system). Может ли студент изменить тему курсовой работы? Может – в соответствии с Порядком оформления курсовых и выпускных квалификационных работ. С этой целью нужно написать личное заявление на имя руководителя факультета с кратким обоснованием своей просьбы. На заявлении необходимо поставить визы руководителя курсовой работы и академического руководителя. Завизированное заявление передается в учебный офис, который вносит соответствующие изменения. Необходимо помнить, что заявление должно быть подано в учебный офис не позднее, чем за один календарный месяц до установленного срока представления итогового варианта курсовой работы. Может ли студент заменить руководителя курсовой работы? Может – в соответствии с Порядком оформления курсовых и выпускных квалификационных работ . Необходимо написать личное заявление на имя декана факультета с кратким обоснованием своей просьбы. Декан имеет право отклонить просьбу студента о замене руководителя, аргументировав свое решение. В случае согласия завизированное заявление передается в учебный офис. Необходимо помнить, что заявление должно быть подано в учебный офис не позднее, чем за один календарный месяц до установленного срока представления итогового</t>
         </is>
       </c>
-      <c r="K32" t="n">
+      <c r="L32" t="n">
         <v>5</v>
       </c>
-      <c r="L32" t="n">
+      <c r="M32" t="n">
         <v>63</v>
       </c>
-      <c r="M32" t="n">
+      <c r="N32" t="n">
         <v>12.6</v>
       </c>
-      <c r="N32" t="n">
+      <c r="O32" t="n">
         <v>0.8888888888888888</v>
       </c>
-      <c r="O32" t="n">
+      <c r="P32" t="n">
         <v>0.7569844126701355</v>
       </c>
-      <c r="P32" t="n">
+      <c r="Q32" t="n">
         <v>0.2010702341794968</v>
       </c>
-      <c r="Q32" t="n">
+      <c r="R32" t="n">
         <v>0.04194539785385132</v>
       </c>
-      <c r="R32" t="n">
+      <c r="S32" t="n">
         <v>33.29560651190951</v>
       </c>
-      <c r="S32" t="n">
+      <c r="T32" t="n">
         <v>0.6562385559082031</v>
       </c>
-      <c r="T32" t="n">
+      <c r="U32" t="n">
         <v>0.4321623742580414</v>
       </c>
-      <c r="U32" t="n">
+      <c r="V32" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W32" t="n">
+        <v>0.3607011437416077</v>
+      </c>
+      <c r="X32" t="n">
         <v>4.149924</v>
       </c>
     </row>
@@ -3114,48 +3470,59 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
+          <t>['Деньги', 'Социальные вопросы', 'Общежития', 'Общежития', 'Деньги', 'Социальные вопросы', 'Общежития', 'Деньги', 'Общежития']</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
           <t>Чтобы получить место в общежитии НИУ ВШЭ, вам необходимо внести соответствующую отметку в пакет документов абитуриента при подаче заявления. Это можно сделать до 25 июля для программ с бюджетными местами и до 15 августа для полностью платных программ. После этого вы сможете увидеть списки рекомендованных к заселению на сайте, начиная с 25 августа. Если вы не попали в списки рекомендованных к заселению, это означает, что вы находитесь в резервном списке и имеете право претендовать на освобождающиеся места в течение учебного года. Информацию о днях заселения можно найти на сайте вместе со списками рекомендованных к заселению. Если вы не успеваете приехать в дни заселения, необходимо уведомить заведующего общежитием о продлении бронирования вашего места. При заселении в общежитие вам потребуется предъявить паспорт, медицинский полис, копию справки 086-У с отметкой о прохождении флюорографии и другие документы.  Подробнее: https://studyabroad.hse.ru/departure1 https://nnov.hse.ru/dormitory/order https://spb.hse.ru/dormitory/docen https://nnov.hse.ru/dormitory/questions</t>
         </is>
       </c>
-      <c r="I33" t="n">
+      <c r="J33" t="n">
         <v>-1</v>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>, что мне требуется общежитие. Что делать? Внести любые изменения в пакет документов абитуриента, в том числе отметку о необходимости общежития, можно в период подачи заявления: для программ с бюджетными местами в срок до 25 июля, для полностью платных программ — до 15 августа. Где и когда можно увидеть списки рекомендованных к заселению и адрес общежития? Информирование о результатах отбора осуществляется путем размещения списков на сайте начиная с 25 августа. Что делать, если студент не попал в списки рекомендованных к заселению в общежитие? Это означает, что студент попал в резервный список, который подтверждает его право претендовать на высвобождающиеся места в течение учебного года. Когда можно будет заселиться в общежитие, если студент увидел себя в списках рекомендованных к заселению? Информация о днях заселения будет опубликована на сайте вместе со списками рекомендованных к заселению в общежития. Что делать, если студент не успевает приехать в дни заселения (заболел, не было билетов и т.д.)? Не отдадут ли место другому? В такой ситуации необходимо известить заведующего общежитием, до какого дня нужно забронировать место. В противном случае через пять дней после указанной даты заезда место перераспредел регистрацией); Документ, подтверждающий состав семьи / копия из домовой книги (берется в ЖЭКе или ТСЖ); Скан справки о доходах по форме 2-НДФЛ за 6 месяцев текущего года всех работающих членов семьи, справки о размере пенсии из ПФР (для пенсионеров), справки из Центра занятости (для безработных). При заселении в общежитие при себе необходимо иметь: Паспорт и его копию Медицинский полис и его копию Копию справки 086-У с отметкой о прохождении флюорографии (ВНИМАНИЕ! Прежде чем отдать оригинал справки в Приемную комиссию, необходимо сделать копию для заселения в общежитие) Студенты, которые не достигли совершеннолетия, в том числе несовершеннолетние дети-сироты, должны оформлять все необходимые документы в присутствии законного представителя или опекуна, либо предоставить согласие законного представителя или опекуна на заключение найма жилого помещения и регистрации по месту пребывания. Согласие на заключение найма жилого помещения (PDF, 471 Кб) Подать документы</t>
         </is>
       </c>
-      <c r="K33" t="n">
+      <c r="L33" t="n">
         <v>8</v>
       </c>
-      <c r="L33" t="n">
+      <c r="M33" t="n">
         <v>135</v>
       </c>
-      <c r="M33" t="n">
+      <c r="N33" t="n">
         <v>16.875</v>
       </c>
-      <c r="N33" t="n">
+      <c r="O33" t="n">
         <v>0.7111111111111111</v>
       </c>
-      <c r="O33" t="n">
+      <c r="P33" t="n">
         <v>0.8823732733726501</v>
       </c>
-      <c r="P33" t="n">
+      <c r="Q33" t="n">
         <v>0.04480961710214615</v>
       </c>
-      <c r="Q33" t="n">
+      <c r="R33" t="n">
         <v>0.07281717658042908</v>
       </c>
-      <c r="R33" t="n">
+      <c r="S33" t="n">
         <v>39.90671886758372</v>
       </c>
-      <c r="S33" t="n">
+      <c r="T33" t="n">
         <v>0.7224839925765991</v>
       </c>
-      <c r="T33" t="n">
+      <c r="U33" t="n">
         <v>0.4941227734088898</v>
       </c>
-      <c r="U33" t="n">
+      <c r="V33" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="W33" t="n">
+        <v>0.3584529757499695</v>
+      </c>
+      <c r="X33" t="n">
         <v>5.741731</v>
       </c>
     </row>
@@ -3197,48 +3564,59 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
+          <t>['Деньги', 'Социальные вопросы', 'Общежития', 'Общежития', 'Деньги', 'Социальные вопросы', 'Общежития', 'Деньги', 'Общежития', 'Деньги', 'Социальные вопросы', 'Общежития', 'Деньги', 'Общежития', 'Деньги', 'Социальные вопросы', 'Общежития', 'Деньги', 'Социальные вопросы', 'Общежития']</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
           <t>Чтобы получить место в общежитии НИУ ВШЭ, вам необходимо внести соответствующую отметку в пакет документов абитуриента при подаче заявления. Это можно сделать до 25 июля для программ с бюджетными местами и до 15 августа для полностью платных программ. После этого вы сможете увидеть списки рекомендованных к заселению на сайте, начиная с 25 августа. Если вы не попали в списки рекомендованных к заселению, это означает, что вы находитесь в резервном списке и имеете право претендовать на освобождающиеся места в течение учебного года. Информацию о днях заселения можно найти на сайте вместе со списками рекомендованных к заселению. Если вы не успеваете приехать в дни заселения, необходимо уведомить заведующего общежитием о продлении бронирования вашего места. При заселении в общежитие вам потребуется предъявить паспорт, медицинский полис, копию справки 086-У с отметкой о прохождении флюорографии и другие документы.  Подробнее: https://studyabroad.hse.ru/departure1 https://nnov.hse.ru/dormitory/order https://spb.hse.ru/dormitory/docen https://nnov.hse.ru/dormitory/questions</t>
         </is>
       </c>
-      <c r="I34" t="n">
+      <c r="J34" t="n">
         <v>1</v>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>, что мне требуется общежитие. Что делать? Внести любые изменения в пакет документов абитуриента, в том числе отметку о необходимости общежития, можно в период подачи заявления: для программ с бюджетными местами в срок до 25 июля, для полностью платных программ — до 15 августа. Где и когда можно увидеть списки рекомендованных к заселению и адрес общежития? Информирование о результатах отбора осуществляется путем размещения списков на сайте начиная с 25 августа. Что делать, если студент не попал в списки рекомендованных к заселению в общежитие? Это означает, что студент попал в резервный список, который подтверждает его право претендовать на высвобождающиеся места в течение учебного года. Когда можно будет заселиться в общежитие, если студент увидел себя в списках рекомендованных к заселению? Информация о днях заселения будет опубликована на сайте вместе со списками рекомендованных к заселению в общежития. Что делать, если студент не успевает приехать в дни заселения (заболел, не было билетов и т.д.)? Не отдадут ли место другому? В такой ситуации необходимо известить заведующего общежитием, до какого дня нужно забронировать место. В противном случае через пять дней после указанной даты заезда место перераспредел регистрацией); Документ, подтверждающий состав семьи / копия из домовой книги (берется в ЖЭКе или ТСЖ); Скан справки о доходах по форме 2-НДФЛ за 6 месяцев текущего года всех работающих членов семьи, справки о размере пенсии из ПФР (для пенсионеров), справки из Центра занятости (для безработных). При заселении в общежитие при себе необходимо иметь: Паспорт и его копию Медицинский полис и его копию Копию справки 086-У с отметкой о прохождении флюорографии (ВНИМАНИЕ! Прежде чем отдать оригинал справки в Приемную комиссию, необходимо сделать копию для заселения в общежитие) Студенты, которые не достигли совершеннолетия, в том числе несовершеннолетние дети-сироты, должны оформлять все необходимые документы в присутствии законного представителя или опекуна, либо предоставить согласие законного представителя или опекуна на заключение найма жилого помещения и регистрации по месту пребывания. Согласие на заключение найма жилого помещения (PDF, 471 Кб) Подать документы , что мне требуется общежитие. Что делать? Внести любые изменения в пакет документов абитуриента, в том числе отметку о необходимости общежития, можно в период подачи заявления: для программ с бюджетными местами в срок до 25 июля, для полностью платных программ — до 15 августа. Где и когда можно увидеть списки рекомендованных к заселению и адрес общежития? Информирование о результатах отбора осуществляется путем размещения списков на сайте начиная с 25 августа. Что делать, если студент не попал в списки рекомендованных к заселению в общежитие? Это означает, что студент попал в резервный список, который подтверждает его право претендовать на высвобождающиеся места в течение учебного года. Когда можно будет заселиться в общежитие, если студент увидел себя в списках рекомендованных к заселению? Информация о днях заселения будет опубликована на сайте вместе со списками рекомендованных к заселению в общежития. Что делать, если студент не успевает приехать в дни заселения (заболел, не было билетов и т.д.)? Не отдадут ли место другому? В такой ситуации необходимо известить заведующего общежитием, до какого дня нужно забронировать место. В противном случае через пять дней после указанной даты заезда место перераспределп – нормированная на диапазон от «0» до «1» сумма баллов ЕГЭ, указанная при поступлении для абитуриентов бакалавриата, нормированная на диапазон от «0» до «1» сумма баллов за вступительные экзамены для абитуриентов магистратуры; нормированные на диапазон от «0» до «1» показатели текущей успеваемости (для студентов бакалавриата, специалитета и магистратуры). Кмат.пол - нормированный на диапазон от «0» до «1» уровень материального положения кандидата на предоставление места в общежитии. Красст - нормированное на диапазон от «0» до «1» расстояние между городом Нижним Новгородом и местом жительства кандидата на предоставление места в общежитии (в километрах). При этом, для всех коэффициентов «1» присваивается максимальной величине показателя, «0» присваивается минимальной величине показателя. Для коэффициента Кмат.пол «1» присваивается также, если документы о доходах не представлены. Обучающиеся и иные лица, нуждающиеся в предоставлении жилого помещения в общежитии НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) – Нижний Новгород по своему усмотрению вправ</t>
         </is>
       </c>
-      <c r="K34" t="n">
+      <c r="L34" t="n">
         <v>8</v>
       </c>
-      <c r="L34" t="n">
+      <c r="M34" t="n">
         <v>135</v>
       </c>
-      <c r="M34" t="n">
+      <c r="N34" t="n">
         <v>16.875</v>
       </c>
-      <c r="N34" t="n">
+      <c r="O34" t="n">
         <v>0.7111111111111111</v>
       </c>
-      <c r="O34" t="n">
+      <c r="P34" t="n">
         <v>0.8828914165496826</v>
       </c>
-      <c r="P34" t="n">
+      <c r="Q34" t="n">
         <v>0.01344216428697109</v>
       </c>
-      <c r="Q34" t="n">
+      <c r="R34" t="n">
         <v>0.1036664843559265</v>
       </c>
-      <c r="R34" t="n">
+      <c r="S34" t="n">
         <v>23.93441831971837</v>
       </c>
-      <c r="S34" t="n">
+      <c r="T34" t="n">
         <v>0.6823767423629761</v>
       </c>
-      <c r="T34" t="n">
+      <c r="U34" t="n">
         <v>0.4941227734088898</v>
       </c>
-      <c r="U34" t="n">
+      <c r="V34" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0.3584529757499695</v>
+      </c>
+      <c r="X34" t="n">
         <v>3.641387</v>
       </c>
     </row>
@@ -3280,44 +3658,55 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Дополнительное образование', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Учебный процесс']</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы?  Подробнее: https://www.hse.ru/science/HSEconf https://www.hse.ru/science/news/announcements/ https://studscience.hse.ru/science\_seance https://studscience.hse.ru/external\_activity</t>
         </is>
       </c>
-      <c r="I35" t="n">
+      <c r="J35" t="n">
         <v>-1</v>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="n">
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="n">
         <v>4</v>
       </c>
-      <c r="L35" t="n">
+      <c r="M35" t="n">
         <v>22</v>
       </c>
-      <c r="M35" t="n">
+      <c r="N35" t="n">
         <v>5.5</v>
       </c>
-      <c r="N35" t="n">
+      <c r="O35" t="n">
         <v>0.9545454545454546</v>
       </c>
-      <c r="O35" t="n">
+      <c r="P35" t="n">
         <v>0.07619420439004898</v>
       </c>
-      <c r="P35" t="n">
+      <c r="Q35" t="n">
         <v>0.3433757126331329</v>
       </c>
-      <c r="Q35" t="n">
+      <c r="R35" t="n">
         <v>0.5804300904273987</v>
       </c>
-      <c r="R35" t="n">
+      <c r="S35" t="n">
         <v>0</v>
       </c>
-      <c r="S35" t="n">
+      <c r="T35" t="n">
         <v>0.09424427151679993</v>
       </c>
-      <c r="T35" t="n">
+      <c r="U35" t="n">
         <v>0.5219830870628357</v>
       </c>
-      <c r="U35" t="n">
+      <c r="V35" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="W35" t="n">
+        <v>0.5202603340148926</v>
+      </c>
+      <c r="X35" t="n">
         <v>3.201099</v>
       </c>
     </row>
@@ -3359,48 +3748,59 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Дополнительное образование', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Учебный процесс', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Социальные вопросы', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Дополнительное образование']</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы?  Подробнее: https://www.hse.ru/science/HSEconf https://www.hse.ru/science/news/announcements/ https://studscience.hse.ru/science\_seance https://studscience.hse.ru/external\_activity</t>
         </is>
       </c>
-      <c r="I36" t="n">
+      <c r="J36" t="n">
         <v>-1</v>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>еваемости студентов) от 01.02.2024 вcтупила в силу 1 марта 2024 года . В большинстве случаев новые возможности повторного изучения дисциплин применяются к периоду пересдач по итогам 3-4 модулей 2023/24 учебного года — в сентябре 2024 года. Приложение к ПОПАТКУС (Положения о промежуточной аттестации и текущем контроле успеваемости студентов), регулирующее особенности обучения в МИЭФ ( Приложение 11. Особенности организации промежуточной аттестации в Международном институте экономики и финансов НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) ) действует до 16 октября 2024 года. 1 сентября 2024 года — дата, после которой для всех студентов, за исключением студентов выпускного курса (20 % примерно, из которых около 5 % потенциально могут иметь задолженности по итогам 3-го модуля, то есть всего таких студентов 1% от общего контингента студентов) будут актуальны новые правила в части принятия решения о сценарии участия в пересдачах и повторном обучении. Для 1% студентов , не справившихся с освоением дисциплин на выпускном курсе, и для студентов, которые должны принять участие во второй пересда сессий указанного периода. Для студентов, не явившихся на экзамен, либо получивших неудовлетворительные оценки - учитываются нули за соответствующие элементы учебного плана. Рейтинг после пересдач рассчитывается с оценками, полученными на пересдачах. Когда публикуются рейтинги Рейтинговые таблицы готовятся после летней и зимней сессий, а также после периодов пересдач Рейтинги различных видов доводятся до сведения студентов в течение текущего учебного года не позднее указанных сроков: Текущий рейтинг до пересдач за 1-ое полугодие – 20 января; Текущий рейтинг после пересдач за 1-ое полугодие – 05 марта; Текущий рейтинг до пересдач за 2-ое полугодие – 15 июля; Текущий рейтинг после пересдач за 2-ое полугодие - 25 октября; Кумулятивный рейтинг – 10 марта и 30 октября. Как увидеть свою позицию в рейтинге Рейтинговые таблицы публикуются не позднее сроков, указанных выше, в открытом доступе на сайтах образовательных программ в разделе Студентам - Рейтинги. На что влияет место в рейтинге Рейтинговая позиция часто используется для распределения различных студенческих благ. Ст</t>
         </is>
       </c>
-      <c r="K36" t="n">
+      <c r="L36" t="n">
         <v>4</v>
       </c>
-      <c r="L36" t="n">
+      <c r="M36" t="n">
         <v>22</v>
       </c>
-      <c r="M36" t="n">
+      <c r="N36" t="n">
         <v>5.5</v>
       </c>
-      <c r="N36" t="n">
+      <c r="O36" t="n">
         <v>0.9545454545454546</v>
       </c>
-      <c r="O36" t="n">
+      <c r="P36" t="n">
         <v>0.7937179207801819</v>
       </c>
-      <c r="P36" t="n">
+      <c r="Q36" t="n">
         <v>0.1504725962877274</v>
       </c>
-      <c r="Q36" t="n">
+      <c r="R36" t="n">
         <v>0.05580946430563927</v>
       </c>
-      <c r="R36" t="n">
+      <c r="S36" t="n">
         <v>3.932373214896296</v>
       </c>
-      <c r="S36" t="n">
+      <c r="T36" t="n">
         <v>0.4630668759346008</v>
       </c>
-      <c r="T36" t="n">
+      <c r="U36" t="n">
         <v>0.5219830870628357</v>
       </c>
-      <c r="U36" t="n">
+      <c r="V36" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="W36" t="n">
+        <v>0.5202603340148926</v>
+      </c>
+      <c r="X36" t="n">
         <v>3.282751</v>
       </c>
     </row>
@@ -3442,48 +3842,59 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Дополнительное образование', 'Учебный процесс', 'Английский язык']</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
           <t>Следующая экзаменационная неделя состоится в феврале 2025 года. Точные даты будут определены дополнительно. Следите за объявлениями на официальном сайте НИУ ВШЭ или обратитесь в учебный офис вашей программы для получения более подробной информации.  Подробнее: https://www.hse.ru/studyspravka/new\_regulations https://www.hse.ru/evaluation/#timetable https://www.hse.ru/studyspravka/examsdataculture https://studyabroad.hse.ru/schools/</t>
         </is>
       </c>
-      <c r="I37" t="n">
+      <c r="J37" t="n">
         <v>0</v>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>. Она обязательна для студентов образовательных программ, в учебный план которых она включена, а так же для определяемых приказом координирующего проректора. Независимые экзамены по цифровым компетенциям Даты и язык проведения Даты проведения Независимые экзамены по цифровым компетенциям проводятся в две волны в 3 и 4 модуле в зависимости от учебного плана конкретной образовательной программы. Приказ Об организации и проведении независимых экзаменов и пересдач независимых экзаменов по цифровым компетенциям для студентов бакалавриата и специалитета в 2024-2025 учебном году 3 модуль Независимый экзамен по цифровым компетенциям для студентов бакалавриата и специалитета в 2024/2025 учебном году начнет проводиться с 1 февраля 2025 года. Первая пересдача по Независимым экзаменам по цифровым компетенциям пройдет с 3 по 7 марта. Вторая пересдача по Независимым экзаменам по цифровым компетенциям пройдет с 19 по 21 марта. Если студенты по уважительной причине пропустят одну из пересдач в марте, для них будет следующая возможность пересдать экзамен в следующий период пересдач: сентябрь- октябрь следующего учебного года. У студентов есть возможность отложить вторую пересПАТКУС (Положения о промежуточной аттестации и текущем контроле успеваемости студентов) от 01.02.2024 Редакция от 01.02.2024 Положения об организации промежуточной аттестации и текущего контроля успеваемости студентов НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) (ПОПАТКУС (Положения о промежуточной аттестации и текущем контроле успеваемости студентов)) вызвала много дискуссий и породила слухи в студенческой среде. Ниже опубликованы ответы на наиболее частно задаваемые вопросы о новой редакции , в том числе конкретные вопросы студентов . С какого момента действует редакция ПОПАТКУС (Положения о промежуточной аттестации и текущем контроле успеваемости студентов) от 01.02.2024? Как долго будут работать "старые" правила и какие именно? Редакция ПОПАТКУС (Положения о промежуточной аттестации и текущем контроле успеваемости студентов) от 01.02.2024 вcтупила в силу 1 марта 2024 года . В большинстве случаев новые возможности повторного изучения дисциплин применяются к периоду пересдач по итогам</t>
         </is>
       </c>
-      <c r="K37" t="n">
+      <c r="L37" t="n">
         <v>4</v>
       </c>
-      <c r="L37" t="n">
+      <c r="M37" t="n">
         <v>34</v>
       </c>
-      <c r="M37" t="n">
+      <c r="N37" t="n">
         <v>8.5</v>
       </c>
-      <c r="N37" t="n">
+      <c r="O37" t="n">
         <v>0.9705882352941176</v>
       </c>
-      <c r="O37" t="n">
+      <c r="P37" t="n">
         <v>0.8494983315467834</v>
       </c>
-      <c r="P37" t="n">
+      <c r="Q37" t="n">
         <v>0.1026047840714455</v>
       </c>
-      <c r="Q37" t="n">
+      <c r="R37" t="n">
         <v>0.04789683595299721</v>
       </c>
-      <c r="R37" t="n">
+      <c r="S37" t="n">
         <v>8.169952791321954</v>
       </c>
-      <c r="S37" t="n">
+      <c r="T37" t="n">
         <v>0.5367122888565063</v>
       </c>
-      <c r="T37" t="n">
+      <c r="U37" t="n">
         <v>0.3921535611152649</v>
       </c>
-      <c r="U37" t="n">
+      <c r="V37" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="W37" t="n">
+        <v>0.4737597107887268</v>
+      </c>
+      <c r="X37" t="n">
         <v>3.493249</v>
       </c>
     </row>
@@ -3525,44 +3936,55 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Дополнительное образование', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Учебный процесс']</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
           <t>Следующая сессия, вероятно, состоится в сентябре 2024 года, так как новые возможности повторного изучения дисциплин обычно применяются к периоду пересдач по итогам 3-4 модулей 2023/24 учебного года. Однако, точные даты могут зависеть от конкретного учебного плана и программы. Рекомендую обратиться в учебный офис вашей программы для получения более точной информации.  Подробнее: https://www.hse.ru/science/HSEconf https://www.hse.ru/science/news/announcements/ https://studscience.hse.ru/external\_activity</t>
         </is>
       </c>
-      <c r="I38" t="n">
+      <c r="J38" t="n">
         <v>-1</v>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="n">
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="n">
         <v>4</v>
       </c>
-      <c r="L38" t="n">
+      <c r="M38" t="n">
         <v>53</v>
       </c>
-      <c r="M38" t="n">
+      <c r="N38" t="n">
         <v>13.25</v>
       </c>
-      <c r="N38" t="n">
+      <c r="O38" t="n">
         <v>0.9245283018867925</v>
       </c>
-      <c r="O38" t="n">
+      <c r="P38" t="n">
         <v>0.09141303598880768</v>
       </c>
-      <c r="P38" t="n">
+      <c r="Q38" t="n">
         <v>0.893156886100769</v>
       </c>
-      <c r="Q38" t="n">
+      <c r="R38" t="n">
         <v>0.01543015148490667</v>
       </c>
-      <c r="R38" t="n">
+      <c r="S38" t="n">
         <v>0</v>
       </c>
-      <c r="S38" t="n">
+      <c r="T38" t="n">
         <v>0.04590271413326263</v>
       </c>
-      <c r="T38" t="n">
+      <c r="U38" t="n">
         <v>0.4214208424091339</v>
       </c>
-      <c r="U38" t="n">
+      <c r="V38" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0.3134422898292542</v>
+      </c>
+      <c r="X38" t="n">
         <v>3.702804</v>
       </c>
     </row>
@@ -3604,44 +4026,55 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Дополнительное образование', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Учебный процесс']</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
           <t>Мне кажется неуместно здесь это обсуждать. Моя цель - проконсультировать тебя по вопросам обучения. Может, у тебя есть еще какие-то вопросы?  Подробнее: https://www.hse.ru/science/HSEconf https://www.hse.ru/science/news/announcements/ https://studscience.hse.ru/science\_seance https://studscience.hse.ru/external\_activity</t>
         </is>
       </c>
-      <c r="I39" t="n">
+      <c r="J39" t="n">
         <v>-1</v>
       </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="n">
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="n">
         <v>4</v>
       </c>
-      <c r="L39" t="n">
+      <c r="M39" t="n">
         <v>22</v>
       </c>
-      <c r="M39" t="n">
+      <c r="N39" t="n">
         <v>5.5</v>
       </c>
-      <c r="N39" t="n">
+      <c r="O39" t="n">
         <v>0.9545454545454546</v>
       </c>
-      <c r="O39" t="n">
+      <c r="P39" t="n">
         <v>0.07619420439004898</v>
       </c>
-      <c r="P39" t="n">
+      <c r="Q39" t="n">
         <v>0.3433757126331329</v>
       </c>
-      <c r="Q39" t="n">
+      <c r="R39" t="n">
         <v>0.5804300904273987</v>
       </c>
-      <c r="R39" t="n">
+      <c r="S39" t="n">
         <v>0</v>
       </c>
-      <c r="S39" t="n">
+      <c r="T39" t="n">
         <v>0.09424427151679993</v>
       </c>
-      <c r="T39" t="n">
+      <c r="U39" t="n">
         <v>0.5219830870628357</v>
       </c>
-      <c r="U39" t="n">
+      <c r="V39" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="W39" t="n">
+        <v>0.5202603340148926</v>
+      </c>
+      <c r="X39" t="n">
         <v>3.327633</v>
       </c>
     </row>
@@ -3683,44 +4116,55 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'ГИА', 'Английский язык', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'ВУЦ', 'Учебный процесс', 'ВУЦ', 'Учебный процесс', 'ВУЦ', 'Деньги', 'Учебный процесс', 'ГИА', 'Английский язык', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'ВУЦ']</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
           <t>Документы на военку подавать не требуется, так как в НИУ ВШЭ нет военной кафедры. Вместо нее существует Военный учебный центр, где студенты могут пройти курс военной подготовки на добровольной основе. Отбор кандидатов проводится на конкурсной основе среди студентов 1 курса бакалавриата. Для участия в конкурсе необходимо пройти медицинскую комиссию и профессиональный отбор в военкомате по месту воинского учета. Сроки обучения составляют 1,5 года. После успешного завершения военных сборов, принятия Присяги и получения диплома об окончании университета выпускники Военного учебного центра зачисляются в запас без прохождения службы по призыву. По вопросам поступления и военного обучения обращайтесь по адресу: Сормовское шоссе, 30, ауд.208, 210, тел. 224-14-49.  Подробнее: https://www.hse.ru/studyspravka/plagiat https://www.hse.ru/studyspravka/documents https://www.hse.ru/studyspravka/Otsrochka</t>
         </is>
       </c>
-      <c r="I40" t="n">
+      <c r="J40" t="n">
         <v>-1</v>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="n">
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="n">
         <v>10</v>
       </c>
-      <c r="L40" t="n">
+      <c r="M40" t="n">
         <v>109</v>
       </c>
-      <c r="M40" t="n">
+      <c r="N40" t="n">
         <v>10.9</v>
       </c>
-      <c r="N40" t="n">
+      <c r="O40" t="n">
         <v>0.8440366972477065</v>
       </c>
-      <c r="O40" t="n">
+      <c r="P40" t="n">
         <v>0.01108105294406414</v>
       </c>
-      <c r="P40" t="n">
+      <c r="Q40" t="n">
         <v>0.9241259098052979</v>
       </c>
-      <c r="Q40" t="n">
+      <c r="R40" t="n">
         <v>0.06479299068450928</v>
       </c>
-      <c r="R40" t="n">
+      <c r="S40" t="n">
         <v>0</v>
       </c>
-      <c r="S40" t="n">
+      <c r="T40" t="n">
         <v>0.05385325849056244</v>
       </c>
-      <c r="T40" t="n">
+      <c r="U40" t="n">
         <v>0.37613844871521</v>
       </c>
-      <c r="U40" t="n">
+      <c r="V40" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="W40" t="n">
+        <v>0.161435604095459</v>
+      </c>
+      <c r="X40" t="n">
         <v>4.734104</v>
       </c>
     </row>
@@ -3762,48 +4206,59 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование']</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
           <t>Чтобы получить справку об обучении в НИУ ВШЭ, нужно обратиться в учебный офис своей образовательной программы. Справка должна быть актуальной (не старше 30 дней на момент подачи заявки) и содержать результаты промежуточной аттестации на момент подачи заявки. Она изготавливается на бланке образовательной организации и содержит информацию о годе поступления, номере и дате приказа о зачислении, текущем статусе студента и перечне изученных дисциплин с указанием полученных оценок и объема в зачетных единицах.  Подробнее: https://spb.hse.ru/hr https://www.hse.ru/studyspravka/transfer</t>
         </is>
       </c>
-      <c r="I41" t="n">
+      <c r="J41" t="n">
         <v>-1</v>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>уки РФ от 12.07.2021 №607 . Справка должна быть актуальной (не старше 30 дней на момент подачи заявки) и содержать результаты промежуточной аттестации на момент подачи заявки. Справка об обучении (она же «Справка об обучении», «Справка о периоде обучения», «Справка об обучении и (или) о периоде обучения», «Академическая справка») как правило изготавливается на бланке образовательной организации и содержит следующую информацию: в каком году и на основании какого документа студент поступил в образовательную организацию; номер и дата приказа о зачислении; текущий статус студента; перечень всех изученных дисциплин и других элементов учебного плана с указанием полученных оценок и объема в зачетных единицах. Студентам зарубежных образовательных организаций: транскрипт (справка об обучении) со статусом студента и перечнем изученных дисциплин с их весом в кредитах за подписью уполномоченного лица. О процедуре признания иностранного образования Если документ об образовании получен в иностранном государстве, то необходимо пройти процедуру признания иностранного образования. Существует два варианта прохождения этой процедуры: I. Свидетельство о признании иностранного образования, выданное Рособрнадзором: Для</t>
         </is>
       </c>
-      <c r="K41" t="n">
+      <c r="L41" t="n">
         <v>4</v>
       </c>
-      <c r="L41" t="n">
+      <c r="M41" t="n">
         <v>72</v>
       </c>
-      <c r="M41" t="n">
+      <c r="N41" t="n">
         <v>18</v>
       </c>
-      <c r="N41" t="n">
+      <c r="O41" t="n">
         <v>0.8194444444444444</v>
       </c>
-      <c r="O41" t="n">
+      <c r="P41" t="n">
         <v>0.7041999697685242</v>
       </c>
-      <c r="P41" t="n">
+      <c r="Q41" t="n">
         <v>0.1639191657304764</v>
       </c>
-      <c r="Q41" t="n">
+      <c r="R41" t="n">
         <v>0.1318808794021606</v>
       </c>
-      <c r="R41" t="n">
+      <c r="S41" t="n">
         <v>43.56437328948022</v>
       </c>
-      <c r="S41" t="n">
+      <c r="T41" t="n">
         <v>0.7409608960151672</v>
       </c>
-      <c r="T41" t="n">
+      <c r="U41" t="n">
         <v>0.5063012838363647</v>
       </c>
-      <c r="U41" t="n">
+      <c r="V41" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W41" t="n">
+        <v>0.3616271615028381</v>
+      </c>
+      <c r="X41" t="n">
         <v>4.132681</v>
       </c>
     </row>
@@ -3845,48 +4300,59 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Дополнительное образование']</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
           <t>Расписание сессий в НИУ ВШЭ формируется в системе планирования расписания учебных занятий (РУЗ). За формирование расписания отвечают ответственные работники подразделений, обеспечивающих сопровождение учебного процесса, и сотрудники Центра сервиса "Департамент". Если в расписании отсутствуют некоторые занятия или не прикреплены ссылки к онлайн-занятиям, необходимо обратиться в учебный офис вашей образовательной программы. При обнаружении конфликта в расписании студент может заявить об этом в учебный офис, и менеджер программы подберет новую подходящую дату. Чтобы заявить об уважительной причине отсутствия на занятиях, нужно воспользоваться специальным сервисом.  Подробнее: https://studyabroad.hse.ru/schools/ https://www.hse.ru/studyspravka/ras\_stud</t>
         </is>
       </c>
-      <c r="I42" t="n">
+      <c r="J42" t="n">
         <v>1</v>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>ании с использованием любого из сервисов не отображаются некоторые занятия, отсутствует расписание по некоторым дисциплинам, или не прикреплены ссылки к онлайн-занятиям, необходимо обратиться в учебный офис вашей образовательной программы — контакты сотрудников размещены на странице образовательной программы на портале НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики). В случае выявления проблем работы системы планирования расписания РУЗ (расписания учебных занятий) , комментариев по вопросам дальнейшего развития просьба направлять сообщения на адрес ruz@hse.ru Как и кем формируется расписание учебных занятий В НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) расписание учебных занятий формируется в системе планирования расписания учебных занятий ( РУЗ (расписания учебных занятий) ; доступна только из локальной сети НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики)). За формирование расписания отвечают: ответственные работники подразделений, обеспечивающих сопровождение учебного процесса (диспетчеры) — по дисциплинам учебных планов в соответствии с запланированной нагрузкой преподавателей на департаментах / факультетах / кафедрах; сотрудники Центра Сервиса "Департамент" — по дисциплинам общеуниверситетских проектов</t>
         </is>
       </c>
-      <c r="K42" t="n">
+      <c r="L42" t="n">
         <v>6</v>
       </c>
-      <c r="L42" t="n">
+      <c r="M42" t="n">
         <v>83</v>
       </c>
-      <c r="M42" t="n">
+      <c r="N42" t="n">
         <v>13.83333333333333</v>
       </c>
-      <c r="N42" t="n">
+      <c r="O42" t="n">
         <v>0.8433734939759037</v>
       </c>
-      <c r="O42" t="n">
+      <c r="P42" t="n">
         <v>0.7431845664978027</v>
       </c>
-      <c r="P42" t="n">
+      <c r="Q42" t="n">
         <v>0.1492046266794205</v>
       </c>
-      <c r="Q42" t="n">
+      <c r="R42" t="n">
         <v>0.1076108142733574</v>
       </c>
-      <c r="R42" t="n">
+      <c r="S42" t="n">
         <v>42.45625760984742</v>
       </c>
-      <c r="S42" t="n">
+      <c r="T42" t="n">
         <v>0.7104449272155762</v>
       </c>
-      <c r="T42" t="n">
+      <c r="U42" t="n">
         <v>0.4895794987678528</v>
       </c>
-      <c r="U42" t="n">
+      <c r="V42" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="W42" t="n">
+        <v>0.3495936095714569</v>
+      </c>
+      <c r="X42" t="n">
         <v>4.777111</v>
       </c>
     </row>
@@ -3928,48 +4394,59 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование']</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
           <t>Чтобы получить справку об обучении в НИУ ВШЭ, нужно обратиться в учебный офис своей образовательной программы. Справка должна быть актуальной (не старше 30 дней на момент подачи заявки) и содержать результаты промежуточной аттестации на момент подачи заявки. Она изготавливается на бланке образовательной организации и содержит информацию о годе поступления, номере и дате приказа о зачислении, текущем статусе студента и перечне изученных дисциплин с указанием полученных оценок и объема в зачетных единицах.  Подробнее: https://spb.hse.ru/hr https://www.hse.ru/studyspravka/transfer</t>
         </is>
       </c>
-      <c r="I43" t="n">
+      <c r="J43" t="n">
         <v>-1</v>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>уки РФ от 12.07.2021 №607 . Справка должна быть актуальной (не старше 30 дней на момент подачи заявки) и содержать результаты промежуточной аттестации на момент подачи заявки. Справка об обучении (она же «Справка об обучении», «Справка о периоде обучения», «Справка об обучении и (или) о периоде обучения», «Академическая справка») как правило изготавливается на бланке образовательной организации и содержит следующую информацию: в каком году и на основании какого документа студент поступил в образовательную организацию; номер и дата приказа о зачислении; текущий статус студента; перечень всех изученных дисциплин и других элементов учебного плана с указанием полученных оценок и объема в зачетных единицах. Студентам зарубежных образовательных организаций: транскрипт (справка об обучении) со статусом студента и перечнем изученных дисциплин с их весом в кредитах за подписью уполномоченного лица. О процедуре признания иностранного образования Если документ об образовании получен в иностранном государстве, то необходимо пройти процедуру признания иностранного образования. Существует два варианта прохождения этой процедуры: I. Свидетельство о признании иностранного образования, выданное Рособрнадзором: Для</t>
         </is>
       </c>
-      <c r="K43" t="n">
+      <c r="L43" t="n">
         <v>4</v>
       </c>
-      <c r="L43" t="n">
+      <c r="M43" t="n">
         <v>72</v>
       </c>
-      <c r="M43" t="n">
+      <c r="N43" t="n">
         <v>18</v>
       </c>
-      <c r="N43" t="n">
+      <c r="O43" t="n">
         <v>0.8194444444444444</v>
       </c>
-      <c r="O43" t="n">
+      <c r="P43" t="n">
         <v>0.7041999697685242</v>
       </c>
-      <c r="P43" t="n">
+      <c r="Q43" t="n">
         <v>0.1639191657304764</v>
       </c>
-      <c r="Q43" t="n">
+      <c r="R43" t="n">
         <v>0.1318808794021606</v>
       </c>
-      <c r="R43" t="n">
+      <c r="S43" t="n">
         <v>43.56437328948022</v>
       </c>
-      <c r="S43" t="n">
+      <c r="T43" t="n">
         <v>0.7409608960151672</v>
       </c>
-      <c r="T43" t="n">
+      <c r="U43" t="n">
         <v>0.5063012838363647</v>
       </c>
-      <c r="U43" t="n">
+      <c r="V43" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="W43" t="n">
+        <v>0.3616271615028381</v>
+      </c>
+      <c r="X43" t="n">
         <v>4.086247</v>
       </c>
     </row>
@@ -4011,48 +4488,59 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Учебный процесс', 'Цифровые системы', 'Обратная связь']</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
           <t>Расписание сессий можно найти на сайте НИУ ВШЭ в разделе "Расписание" на странице образовательной программы вашей академической группы. Также расписание может быть доступно в едином личном кабинете студента и в приложении HSE App X. Если у вас возникают проблемы с поиском расписания или конфликты в расписании, рекомендуется обратиться к администратору программы или воспользоваться технической поддержкой.  Подробнее: https://electives.hse.ru/sw https://www.hse.ru/studyspravka/ras\_stud</t>
         </is>
       </c>
-      <c r="I44" t="n">
+      <c r="J44" t="n">
         <v>-1</v>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>Расписание занятий Расписание учебных занятий студентов Где найти расписание По академический группе : на странице образовательной программы на портале НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики), где в разделе «Расписание» выводится информация обо всех дисциплинах, которые включены в индивидуальные учебные планы студентов каждой группы; на сайте системы планирования расписания учебных занятий ( РУЗ (расписания учебных занятий) ; доступна только из локальной сети НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики)). Индивидуальное : в едином личном кабинете ( ЕЛК (единый личный кабинет) ) студента в разделе «Расписание»; на сайте системы планирования расписания учебных занятий ( РУЗ (расписания учебных занятий) ; доступна только из локальной сети НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики)); в приложении HSE App X, которое можно скачать в App Store , Google Play и AppGallery , можно: осуществлять поиск занятий по преподавателям или академическим группам студентов; ознакомиться с местоположением корпуса, где запланировано занятие; интегрировать занятия в личный календарь. Если обнаружен конфликт в расписании Дисциплин учебного плана : можно либо перевестись в другую учебную группу волны; дисциплины, у которых нет составленного или подходящего вам по ограничениям расписания и заявки на которые были направлены во время 1 волны. Для отзыва заявки в разделе "Мои заявки" необходимо: поставить галочку в чек-бокс справа в строке с нужной заявкой нажать кнопку "Отозвать заявку" подтвердить действие во всплывающих окнах. Раздел «Моё расписание» Для перехода к разделу необходимо в левой части экрана выбрать раздел "Мое расписание" В разделе отображен экран просмотра вашего расписания: назначенного в учетной системе или по итогам выбора в предыдущую кампанию выбранного в текущую кампанию во время 2 волны В расписании выводятся: рядом с названием месяца - количество пересечений в данном месяце желтым цветом строки с пересекающимся расписанием, т.е. занятия по разным дисциплинам начинаются в одно время. Около дня будет выведен знак</t>
         </is>
       </c>
-      <c r="K44" t="n">
+      <c r="L44" t="n">
         <v>4</v>
       </c>
-      <c r="L44" t="n">
+      <c r="M44" t="n">
         <v>56</v>
       </c>
-      <c r="M44" t="n">
+      <c r="N44" t="n">
         <v>14</v>
       </c>
-      <c r="N44" t="n">
+      <c r="O44" t="n">
         <v>0.8571428571428571</v>
       </c>
-      <c r="O44" t="n">
+      <c r="P44" t="n">
         <v>0.7331405878067017</v>
       </c>
-      <c r="P44" t="n">
+      <c r="Q44" t="n">
         <v>0.156537726521492</v>
       </c>
-      <c r="Q44" t="n">
+      <c r="R44" t="n">
         <v>0.1103216484189034</v>
       </c>
-      <c r="R44" t="n">
+      <c r="S44" t="n">
         <v>18.23559683796628</v>
       </c>
-      <c r="S44" t="n">
+      <c r="T44" t="n">
         <v>0.6310037970542908</v>
       </c>
-      <c r="T44" t="n">
+      <c r="U44" t="n">
         <v>0.4554103016853333</v>
       </c>
-      <c r="U44" t="n">
+      <c r="V44" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="W44" t="n">
+        <v>0.2738432884216309</v>
+      </c>
+      <c r="X44" t="n">
         <v>3.865264</v>
       </c>
     </row>
@@ -4094,48 +4582,59 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов']</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
           <t>Для досрочной сдачи сессии необходимо обратиться к менеджеру своей образовательной программы для возможного изменения расписания или подать заявку о переносе одного из экзаменов на другое время не позднее трех дней до начала сессии. Если вы находитесь в академическом отпуске, вы можете досрочно выйти из него, подав заявление о выходе из отпуска до окончания периода времени, на который он был предоставлен, и получить допуск к учебному процессу. Если у вас есть дополнительные вопросы по этой теме, пожалуйста, уточните их.  Подробнее: https://studyabroad.hse.ru/schools/ https://www.hse.ru/studyspravka/ras\_stud</t>
         </is>
       </c>
-      <c r="I45" t="n">
+      <c r="J45" t="n">
         <v>1</v>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>с местоположением корпуса, где запланировано занятие; интегрировать занятия в личный календарь. Если обнаружен конфликт в расписании Дисциплин учебного плана : можно либо перевестись в другую учебную группу в рамках одной дисциплины, либо, если группа только одна, можно заменить одну из вариативных дисциплин на другую, с более подходящим расписанием — обратитесь к менеджеру своей образовательной программы за консультацией. Экзаменов на сессии : если в расписании сессии в день стоит несколько экзаменов (включая повторные сдачи блокирующих в течение 10 дней до сессии), то можно либо сдавать несколько экзаменов в один день, если по времени не пересекаются (в этом случае нельзя апеллировать к процедуре экзамена), либо подать заявку о переносе одного из экзаменов на другое время не позднее трех дней до начала сессии. Пересдач с расписанием занятий : подайте заявку для изменения имеющейся даты пересдачи не позднее трех дней до начала периода пересдач по графику учебного процесса . Если возникли проблемы с расписанием Если в расписании с использованием любого из сервисов не отображаются некоторые занятия, отсутствует расписание по некоторым дисциплинам, или не прикреплены ссылки к онлайн-занятиям, необходимо обратиться в учебный офис вашей образовательной программы — контак</t>
         </is>
       </c>
-      <c r="K45" t="n">
+      <c r="L45" t="n">
         <v>4</v>
       </c>
-      <c r="L45" t="n">
+      <c r="M45" t="n">
         <v>79</v>
       </c>
-      <c r="M45" t="n">
+      <c r="N45" t="n">
         <v>19.75</v>
       </c>
-      <c r="N45" t="n">
+      <c r="O45" t="n">
         <v>0.8734177215189873</v>
       </c>
-      <c r="O45" t="n">
+      <c r="P45" t="n">
         <v>0.8568710088729858</v>
       </c>
-      <c r="P45" t="n">
+      <c r="Q45" t="n">
         <v>0.09472200274467468</v>
       </c>
-      <c r="Q45" t="n">
+      <c r="R45" t="n">
         <v>0.04840692132711411</v>
       </c>
-      <c r="R45" t="n">
+      <c r="S45" t="n">
         <v>30.93315413884446</v>
       </c>
-      <c r="S45" t="n">
+      <c r="T45" t="n">
         <v>0.6470115780830383</v>
       </c>
-      <c r="T45" t="n">
+      <c r="U45" t="n">
         <v>0.3908182084560394</v>
       </c>
-      <c r="U45" t="n">
+      <c r="V45" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0.3403014838695526</v>
+      </c>
+      <c r="X45" t="n">
         <v>4.024553</v>
       </c>
     </row>
@@ -4177,48 +4676,59 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Деньги', 'Учебный процесс', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов']</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
           <t>Я могу ответить на ваш вопрос только частично. В НИУ ВШЭ студент может быть отчислен по нескольким причинам, включая недобросовестное освоение образовательной программы и невыполнение учебного плана. Если студент получает академические задолженности по трем и более дисциплинам по итогам промежуточной аттестации, он может быть отчислен. Решение об отчислении принимает проректор университета. Что касается досрочной сдачи сессии, вы можете обратиться к менеджеру своей образовательной программы за консультацией. Вы также можете подать заявку о переносе одного из экзаменов на другое время не позднее трех дней до начала сессии. Для получения более подробной информации рекомендую обратиться в учебный офис вашей образовательной программы.  Подробнее: https://studyabroad.hse.ru/schools/ https://www.hse.ru/studyspravka/ras\_stud</t>
         </is>
       </c>
-      <c r="I46" t="n">
+      <c r="J46" t="n">
         <v>0</v>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>с местоположением корпуса, где запланировано занятие; интегрировать занятия в личный календарь. Если обнаружен конфликт в расписании Дисциплин учебного плана : можно либо перевестись в другую учебную группу в рамках одной дисциплины, либо, если группа только одна, можно заменить одну из вариативных дисциплин на другую, с более подходящим расписанием — обратитесь к менеджеру своей образовательной программы за консультацией. Экзаменов на сессии : если в расписании сессии в день стоит несколько экзаменов (включая повторные сдачи блокирующих в течение 10 дней до сессии), то можно либо сдавать несколько экзаменов в один день, если по времени не пересекаются (в этом случае нельзя апеллировать к процедуре экзамена), либо подать заявку о переносе одного из экзаменов на другое время не позднее трех дней до начала сессии. Пересдач с расписанием занятий : подайте заявку для изменения имеющейся даты пересдачи не позднее трех дней до начала периода пересдач по графику учебного процесса . Если возникли проблемы с расписанием Если в расписании с использованием любого из сервисов не отображаются некоторые занятия, отсутствует расписание по некоторым дисциплинам, или не прикреплены ссылки к онлайн-занятиям, необходимо обратиться в учебный офис вашей образовательной программы — контак</t>
         </is>
       </c>
-      <c r="K46" t="n">
+      <c r="L46" t="n">
         <v>8</v>
       </c>
-      <c r="L46" t="n">
+      <c r="M46" t="n">
         <v>100</v>
       </c>
-      <c r="M46" t="n">
+      <c r="N46" t="n">
         <v>12.5</v>
       </c>
-      <c r="N46" t="n">
+      <c r="O46" t="n">
         <v>0.82</v>
       </c>
-      <c r="O46" t="n">
+      <c r="P46" t="n">
         <v>0.8938616514205933</v>
       </c>
-      <c r="P46" t="n">
+      <c r="Q46" t="n">
         <v>0.07884019613265991</v>
       </c>
-      <c r="Q46" t="n">
+      <c r="R46" t="n">
         <v>0.02729824744164944</v>
       </c>
-      <c r="R46" t="n">
+      <c r="S46" t="n">
         <v>35.83866658233135</v>
       </c>
-      <c r="S46" t="n">
+      <c r="T46" t="n">
         <v>0.6522145867347717</v>
       </c>
-      <c r="T46" t="n">
+      <c r="U46" t="n">
         <v>0.3929842114448547</v>
       </c>
-      <c r="U46" t="n">
+      <c r="V46" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="W46" t="n">
+        <v>0.3784665763378143</v>
+      </c>
+      <c r="X46" t="n">
         <v>4.566511</v>
       </c>
     </row>
@@ -4260,48 +4770,59 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Учебный процесс', 'Цифровые системы', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Учебный процесс', 'Английский язык', 'Учебный процесс', 'Цифровые системы', 'Обратная связь']</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
           <t>Расписание сессий можно найти на сайте НИУ ВШЭ в разделе "Расписание" на странице образовательной программы вашей академической группы. Также расписание может быть доступно в едином личном кабинете студента и в приложении HSE App X. Если у вас возникают проблемы с поиском расписания или конфликты в расписании, рекомендуется обратиться к администратору программы или воспользоваться технической поддержкой.  Подробнее: https://electives.hse.ru/sw https://www.hse.ru/studyspravka/ras\_stud</t>
         </is>
       </c>
-      <c r="I47" t="n">
+      <c r="J47" t="n">
         <v>-1</v>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>Расписание занятий Расписание учебных занятий студентов Где найти расписание По академический группе : на странице образовательной программы на портале НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики), где в разделе «Расписание» выводится информация обо всех дисциплинах, которые включены в индивидуальные учебные планы студентов каждой группы; на сайте системы планирования расписания учебных занятий ( РУЗ (расписания учебных занятий) ; доступна только из локальной сети НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики)). Индивидуальное : в едином личном кабинете ( ЕЛК (единый личный кабинет) ) студента в разделе «Расписание»; на сайте системы планирования расписания учебных занятий ( РУЗ (расписания учебных занятий) ; доступна только из локальной сети НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики)); в приложении HSE App X, которое можно скачать в App Store , Google Play и AppGallery , можно: осуществлять поиск занятий по преподавателям или академическим группам студентов; ознакомиться с местоположением корпуса, где запланировано занятие; интегрировать занятия в личный календарь. Если обнаружен конфликт в расписании Дисциплин учебного плана : можно либо перевестись в другую учебную группу волны; дисциплины, у которых нет составленного или подходящего вам по ограничениям расписания и заявки на которые были направлены во время 1 волны. Для отзыва заявки в разделе "Мои заявки" необходимо: поставить галочку в чек-бокс справа в строке с нужной заявкой нажать кнопку "Отозвать заявку" подтвердить действие во всплывающих окнах. Раздел «Моё расписание» Для перехода к разделу необходимо в левой части экрана выбрать раздел "Мое расписание" В разделе отображен экран просмотра вашего расписания: назначенного в учетной системе или по итогам выбора в предыдущую кампанию выбранного в текущую кампанию во время 2 волны В расписании выводятся: рядом с названием месяца - количество пересечений в данном месяце желтым цветом строки с пересекающимся расписанием, т.е. занятия по разным дисциплинам начинаются в одно время. Около дня будет выведен знак Расписание занятий Расписание учебных занятий студентов Где найти расписание По академический группе : на странице образовательной программы на портале НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики), где в разделе «Расписание» выводится информация обо всех дисциплинах, которые включены в индивидуальные учебные планы студентов каждой группы; на сайте системы планирования расписания учебных занятий ( РУЗ (расписания учебных занятий) ; доступна только из локальной сети НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики)). Индивидуальное : в едином личном кабинете ( ЕЛК (единый личный кабинет) ) студента в разделе «Расписание»; на сайте системы планирования расписания учебных занятий ( РУЗ (расписания учебных занятий) ; доступна только из локальной сети НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики)); в приложении HSE App X, которое можно скачать в App Store , Google Play и AppGallery , можно: осуществлять поиск занятий по преподавателям или академическим группам студентов; ознакомиться с местоположением корпуса, где запланировано занятие; интегрировать занятия в личный календарь. Если обнаружен конфликт в расписании Дисциплин учебного плана : можно либо перевестись в другую учебную группу Заявки на дисциплины могут быть со следующими статусами: Принята — заявка принята; Заявка на рассмотрении - заявка находится на рассмотрении у менеджера Отменена нет мест Отменена — заявка отменена менеджером образовательной программы или системой Включена в ИУП (индивидуальный учебный план) — заявка утверждена. Заявки на расписание могут быть со следующими статусами: Заявка на расписание принята Отменена нет мест Отменена Заявка на расписание отправлена Включена в ИУП (индивидуальный учебный план) Если по дисциплине есть заявки на расписание, то они будут расположены в строках под заявкой на дисциплину. Для их просмотра необходимо развернуть список, нажав на знак: В результате вы увидите полный список заявок на расписание по дисциплине с их текущими статусами. В разделе "Мои заявки": во время 1 волны вы можете отозвать заявки на дисциплину; во время 2 волны вы можете отозвать заявки на: дисциплины и расписания, которые были направлены во время 2 волны; дисциплины, у которых нет составленного или подходящего вам по ограничениям расписания и заявки на которые были направлены во время 1 волны. Для отзыва заявки в разделе "Мои заявки" необходимо: поставить галочку</t>
         </is>
       </c>
-      <c r="K47" t="n">
+      <c r="L47" t="n">
         <v>4</v>
       </c>
-      <c r="L47" t="n">
+      <c r="M47" t="n">
         <v>56</v>
       </c>
-      <c r="M47" t="n">
+      <c r="N47" t="n">
         <v>14</v>
       </c>
-      <c r="N47" t="n">
+      <c r="O47" t="n">
         <v>0.8571428571428571</v>
       </c>
-      <c r="O47" t="n">
+      <c r="P47" t="n">
         <v>0.7729478478431702</v>
       </c>
-      <c r="P47" t="n">
+      <c r="Q47" t="n">
         <v>0.02037646621465683</v>
       </c>
-      <c r="Q47" t="n">
+      <c r="R47" t="n">
         <v>0.206675723195076</v>
       </c>
-      <c r="R47" t="n">
+      <c r="S47" t="n">
         <v>9.907642858055603</v>
       </c>
-      <c r="S47" t="n">
+      <c r="T47" t="n">
         <v>0.596632719039917</v>
       </c>
-      <c r="T47" t="n">
+      <c r="U47" t="n">
         <v>0.4554103016853333</v>
       </c>
-      <c r="U47" t="n">
+      <c r="V47" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="W47" t="n">
+        <v>0.2738432884216309</v>
+      </c>
+      <c r="X47" t="n">
         <v>3.568828</v>
       </c>
     </row>
@@ -4343,48 +4864,59 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Выпускникам', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Учебный процесс', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Обратная связь', 'Безопасность', 'Социальные вопросы']</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
           <t>Каникулы предоставляются студентам после успешного прохождения государственной итоговой аттестации (ГИА). Продолжительность каникул определяется графиком учебного процесса текущего учебного года. В 2024/2025 учебном году каникулы предоставляются до 12 августа. Для подачи заявки на последипломный отпуск студенты должны воспользоваться сервисом "Завершение обучения". Если студент не подаст заявление о предоставлении каникул, то после успешного прохождения ГИА он будет отчислен из университета в связи с завершением обучения.  Подробнее: https://www.hse.ru/studyspravka/igaotpusk https://www.hse.ru/studyspravka/theend https://www.hse.ru/studyspravka/Otsrochka</t>
         </is>
       </c>
-      <c r="I48" t="n">
+      <c r="J48" t="n">
         <v>-1</v>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>Последипломный отпуск Последипломный отпуск после прохождения студентами государственной итоговой аттестации Последипломные каникулы Процедура предоставления Документы Полезные ссылки ГИА (государственная итоговая аттестация) Сервис "Завершение обучения" График учебного процесса Приложение к диплому на английском языке После успешного прохождения государственной итоговой аттестации (далее — ГИА (государственная итоговая аттестация)) студенту могут быть предоставлены каникулы (последипломный отпуск). Продолжительность каникул определяется графиком учебного процесса текущего учебного года . В 2024/2025 уч. году каникулы предоставляются до 12 августа . Процедура предоставления каникул До начала ГИА (государственная итоговая аттестация) каждый студент, завершающий обучение, может подать заявку на последипломный отпуск в сервисе «Завершение обучения» Студенты, не подавшие заявления о предоставлении каникул, после успешного прохождения ГИА (государственная итоговая аттестация), подлежат отчислению из университета в связи с завершением обучения. В отношении студентов, подавших заявление о предоставлении каникул, издается приказ о предоставлении каникул (последипломного отпуска), дата заверш</t>
         </is>
       </c>
-      <c r="K48" t="n">
+      <c r="L48" t="n">
         <v>6</v>
       </c>
-      <c r="L48" t="n">
+      <c r="M48" t="n">
         <v>65</v>
       </c>
-      <c r="M48" t="n">
+      <c r="N48" t="n">
         <v>10.83333333333333</v>
       </c>
-      <c r="N48" t="n">
+      <c r="O48" t="n">
         <v>0.8461538461538461</v>
       </c>
-      <c r="O48" t="n">
+      <c r="P48" t="n">
         <v>0.8028495311737061</v>
       </c>
-      <c r="P48" t="n">
+      <c r="Q48" t="n">
         <v>0.05968851968646049</v>
       </c>
-      <c r="Q48" t="n">
+      <c r="R48" t="n">
         <v>0.1374619454145432</v>
       </c>
-      <c r="R48" t="n">
+      <c r="S48" t="n">
         <v>44.55951757619938</v>
       </c>
-      <c r="S48" t="n">
+      <c r="T48" t="n">
         <v>0.7336074709892273</v>
       </c>
-      <c r="T48" t="n">
+      <c r="U48" t="n">
         <v>0.3054324388504028</v>
       </c>
-      <c r="U48" t="n">
+      <c r="V48" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="W48" t="n">
+        <v>0.3527549505233765</v>
+      </c>
+      <c r="X48" t="n">
         <v>3.940185</v>
       </c>
     </row>
@@ -4426,48 +4958,59 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Выпускникам', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Учебный процесс', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Обратная связь', 'Безопасность', 'Социальные вопросы', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Выпускникам', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Наука', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Обратная связь', 'Безопасность', 'Социальные вопросы', 'Деньги', 'Учебный процесс', 'Социальные вопросы']</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
           <t>Каникулы предоставляются студентам после успешного прохождения государственной итоговой аттестации (ГИА). Продолжительность каникул определяется графиком учебного процесса текущего учебного года. В 2024/2025 учебном году каникулы предоставляются до 12 августа. Для подачи заявки на последипломный отпуск студенты должны воспользоваться сервисом "Завершение обучения". Если студент не подаст заявление о предоставлении каникул, то после успешного прохождения ГИА он будет отчислен из университета в связи с завершением обучения.  Подробнее: https://www.hse.ru/studyspravka/igaotpusk https://www.hse.ru/studyspravka/theend https://www.hse.ru/studyspravka/Otsrochka</t>
         </is>
       </c>
-      <c r="I49" t="n">
+      <c r="J49" t="n">
         <v>-1</v>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>Последипломный отпуск Последипломный отпуск после прохождения студентами государственной итоговой аттестации Последипломные каникулы Процедура предоставления Документы Полезные ссылки ГИА (государственная итоговая аттестация) Сервис "Завершение обучения" График учебного процесса Приложение к диплому на английском языке После успешного прохождения государственной итоговой аттестации (далее — ГИА (государственная итоговая аттестация)) студенту могут быть предоставлены каникулы (последипломный отпуск). Продолжительность каникул определяется графиком учебного процесса текущего учебного года . В 2024/2025 уч. году каникулы предоставляются до 12 августа . Процедура предоставления каникул До начала ГИА (государственная итоговая аттестация) каждый студент, завершающий обучение, может подать заявку на последипломный отпуск в сервисе «Завершение обучения» Студенты, не подавшие заявления о предоставлении каникул, после успешного прохождения ГИА (государственная итоговая аттестация), подлежат отчислению из университета в связи с завершением обучения. В отношении студентов, подавших заявление о предоставлении каникул, издается приказ о предоставлении каникул (последипломного отпуска), дата заверш Последипломный отпуск Последипломный отпуск после прохождения студентами государственной итоговой аттестации Последипломные каникулы Процедура предоставления Документы Полезные ссылки ГИА (государственная итоговая аттестация) Сервис "Завершение обучения" График учебного процесса Приложение к диплому на английском языке После успешного прохождения государственной итоговой аттестации (далее — ГИА (государственная итоговая аттестация)) студенту могут быть предоставлены каникулы (последипломный отпуск). Продолжительность каникул определяется графиком учебного процесса текущего учебного года . В 2024/2025 уч. году каникулы предоставляются до 12 августа . Процедура предоставления каникул До начала ГИА (государственная итоговая аттестация) каждый студент, завершающий обучение, может подать заявку на последипломный отпуск в сервисе «Завершение обучения» Студенты, не подавшие заявления о предоставлении каникул, после успешного прохождения ГИА (государственная итоговая аттестация), подлежат отчислению из университета в связи с завершением обучения. В отношении студентов, подавших заявление о предоставлении каникул, издается приказ о предоставлении каникул (последипломного отпуска), дата заверш</t>
         </is>
       </c>
-      <c r="K49" t="n">
+      <c r="L49" t="n">
         <v>6</v>
       </c>
-      <c r="L49" t="n">
+      <c r="M49" t="n">
         <v>65</v>
       </c>
-      <c r="M49" t="n">
+      <c r="N49" t="n">
         <v>10.83333333333333</v>
       </c>
-      <c r="N49" t="n">
+      <c r="O49" t="n">
         <v>0.8461538461538461</v>
       </c>
-      <c r="O49" t="n">
+      <c r="P49" t="n">
         <v>0.7746724486351013</v>
       </c>
-      <c r="P49" t="n">
+      <c r="Q49" t="n">
         <v>0.02000055834650993</v>
       </c>
-      <c r="Q49" t="n">
+      <c r="R49" t="n">
         <v>0.2053270041942596</v>
       </c>
-      <c r="R49" t="n">
+      <c r="S49" t="n">
         <v>27.61993112253067</v>
       </c>
-      <c r="S49" t="n">
+      <c r="T49" t="n">
         <v>0.6728333234786987</v>
       </c>
-      <c r="T49" t="n">
+      <c r="U49" t="n">
         <v>0.3054324388504028</v>
       </c>
-      <c r="U49" t="n">
+      <c r="V49" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="W49" t="n">
+        <v>0.3527549505233765</v>
+      </c>
+      <c r="X49" t="n">
         <v>3.82027</v>
       </c>
     </row>
@@ -4509,48 +5052,59 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Выпускникам', 'Учебный процесс', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Учебный процесс', 'Цифровые системы']</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
           <t>Каникулы в графике учебного процесса обычно предоставляются после успешного прохождения государственной итоговой аттестации (ГИА). Продолжительность каникул определяется графиком учебного процесса текущего учебного года. В 2024/2025 учебном году каникулы предоставляются до 12 августа. Однако, процедура предоставления каникул требует подачи заявки на последипломный отпуск в сервисе "Завершение обучения" до начала ГИА. Студенты, не подавшие заявления о предоставлении каникул, подлежат отчислению из университета в связи с завершением обучения.  Подробнее: https://www.hse.ru/studyspravka/igaotpusk https://www.hse.ru/studyspravka/theend https://www.hse.ru/docs/799699678.html https://www.hse.ru/studyspravka/grafik</t>
         </is>
       </c>
-      <c r="I50" t="n">
+      <c r="J50" t="n">
         <v>-1</v>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>Последипломный отпуск Последипломный отпуск после прохождения студентами государственной итоговой аттестации Последипломные каникулы Процедура предоставления Документы Полезные ссылки ГИА (государственная итоговая аттестация) Сервис "Завершение обучения" График учебного процесса Приложение к диплому на английском языке После успешного прохождения государственной итоговой аттестации (далее — ГИА (государственная итоговая аттестация)) студенту могут быть предоставлены каникулы (последипломный отпуск). Продолжительность каникул определяется графиком учебного процесса текущего учебного года . В 2024/2025 уч. году каникулы предоставляются до 12 августа . Процедура предоставления каникул До начала ГИА (государственная итоговая аттестация) каждый студент, завершающий обучение, может подать заявку на последипломный отпуск в сервисе «Завершение обучения» Студенты, не подавшие заявления о предоставлении каникул, после успешного прохождения ГИА (государственная итоговая аттестация), подлежат отчислению из университета в связи с завершением обучения. В отношении студентов, подавших заявление о предоставлении каникул, издается приказ о предоставлении каникул (последипломного отпуска), дата завершГрафик учебного процесса Академический календарь (График учебного процесса) Учебный год разбит на 4 модуля, каждый из которых длится от 8 до 12 недель. Точные даты начала и окон\xadчания каждого модуля зависят от выходных и нерабочих праздничных дней в текущем году. Некоторые программы имеют в году два семестра или три модуля Документы График учебного процесса – это документ, определяющий последовательность и чередование обучения, аттестации и каникулярного времени студентов всех направлений и специальностей всех курсов НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) в течение учебного года. График учебного процесса создается и утверждается ежегодно. На графике определены количество учебных модулей в году, количество дней в модулях и каникулярное время. График обязателен для выполнения всеми участниками образовательного процесса. Приказы: Приказ "Об утверждении типового графика учебного процесса на 2024/2025 учебный год" Приказ "Об утверждении типового графика учебного процесса на 2025/2026 учебный год"олняет обязанности, связанные с освоением им образовательной программы, в том числе посещение учебных занятий, предусмотренных индивидуальным учебным планом. Если в течение 10 календарных дней после завершения отпуска обучающийся не приступил к освоению образовательной программы, в том числе не посещает учебные занятия, предусмотренные индивидуальным учебным планом, то он подлежит отчислению за невыполнение обязанностей по добросовестному освоению образовательной программы и выполнению учебного плана. Выход из академического и иных отпусков регламентируется отдельным локальным нормативным актом Университета. 30.11.2022 № 6.18.1-01/301122-1</t>
         </is>
       </c>
-      <c r="K50" t="n">
+      <c r="L50" t="n">
         <v>6</v>
       </c>
-      <c r="L50" t="n">
+      <c r="M50" t="n">
         <v>67</v>
       </c>
-      <c r="M50" t="n">
+      <c r="N50" t="n">
         <v>11.16666666666667</v>
       </c>
-      <c r="N50" t="n">
+      <c r="O50" t="n">
         <v>0.8059701492537313</v>
       </c>
-      <c r="O50" t="n">
+      <c r="P50" t="n">
         <v>0.895763635635376</v>
       </c>
-      <c r="P50" t="n">
+      <c r="Q50" t="n">
         <v>0.03155867382884026</v>
       </c>
-      <c r="Q50" t="n">
+      <c r="R50" t="n">
         <v>0.07267775386571884</v>
       </c>
-      <c r="R50" t="n">
+      <c r="S50" t="n">
         <v>26.5122524831176</v>
       </c>
-      <c r="S50" t="n">
+      <c r="T50" t="n">
         <v>0.6959829926490784</v>
       </c>
-      <c r="T50" t="n">
+      <c r="U50" t="n">
         <v>0.527799665927887</v>
       </c>
-      <c r="U50" t="n">
+      <c r="V50" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="W50" t="n">
+        <v>0.3877084851264954</v>
+      </c>
+      <c r="X50" t="n">
         <v>4.503456</v>
       </c>
     </row>
@@ -4592,48 +5146,59 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Учебный процесс', 'Цифровые системы', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Социальные вопросы']</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
           <t>График учебного процесса - это документ, который определяет последовательность и чередование обучения, аттестации и каникулярного времени студентов всех направлений и специальностей всех курсов НИУ ВШЭ в течение учебного года. Он создается и утверждается ежегодно и является обязательным для выполнения всеми участниками образовательного процесса.  Подробнее: https://www.hse.ru/studyspravka/grafik https://spb.hse.ru/io/studyabroad/overview https://www.hse.ru/studyspravka/ras\_stud</t>
         </is>
       </c>
-      <c r="I51" t="n">
+      <c r="J51" t="n">
         <v>1</v>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>График учебного процесса Академический календарь (График учебного процесса) Учебный год разбит на 4 модуля, каждый из которых длится от 8 до 12 недель. Точные даты начала и окон\xadчания каждого модуля зависят от выходных и нерабочих праздничных дней в текущем году. Некоторые программы имеют в году два семестра или три модуля Документы График учебного процесса – это документ, определяющий последовательность и чередование обучения, аттестации и каникулярного времени студентов всех направлений и специальностей всех курсов НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) в течение учебного года. График учебного процесса создается и утверждается ежегодно. На графике определены количество учебных модулей в году, количество дней в модулях и каникулярное время. График обязателен для выполнения всеми участниками образовательного процесса. Приказы: Приказ "Об утверждении типового графика учебного процесса на 2024/2025 учебный год" Приказ "Об утверждении типового графика учебного процесса на 2025/2026 учебный год"Расписание занятий Расписание учебных занятий студентов Где найти расписание По академический группе : на странице образовательной программы на портале НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики), где в разделе «Расписание» выводится информация обо всех дисциплинах, которые включены в индивидуальные учебные планы студентов каждой группы; на сайте системы планирования расписания учебных занятий ( РУЗ (расписания учебных занятий) ; доступна только из локальной сети НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики)). Индивидуальное : в едином личном кабинете ( ЕЛК (единый личный кабинет) ) студента в разделе «Расписание»; на сайте системы планирования расписания учебных занятий ( РУЗ (расписания учебных занятий) ; доступна только из локальной сети НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики)); в приложении HSE App X, которое можно скачать в App Store , Google Play и AppGallery , можно: осуществлять поиск занятий по преподавателям или академическим группам студентов; ознакомиться с местоположением корпуса, где запланировано занятие; интегрировать занятия в личный календарь. Если обнаружен конфликт в расписании Дисциплин учебного плана : можно либо перевестись в другую учебную группу</t>
         </is>
       </c>
-      <c r="K51" t="n">
+      <c r="L51" t="n">
         <v>3</v>
       </c>
-      <c r="L51" t="n">
+      <c r="M51" t="n">
         <v>43</v>
       </c>
-      <c r="M51" t="n">
+      <c r="N51" t="n">
         <v>14.33333333333333</v>
       </c>
-      <c r="N51" t="n">
+      <c r="O51" t="n">
         <v>0.8372093023255814</v>
       </c>
-      <c r="O51" t="n">
+      <c r="P51" t="n">
         <v>0.8523335456848145</v>
       </c>
-      <c r="P51" t="n">
+      <c r="Q51" t="n">
         <v>0.1102250441908836</v>
       </c>
-      <c r="Q51" t="n">
+      <c r="R51" t="n">
         <v>0.03744141384959221</v>
       </c>
-      <c r="R51" t="n">
+      <c r="S51" t="n">
         <v>21.78431368227939</v>
       </c>
-      <c r="S51" t="n">
+      <c r="T51" t="n">
         <v>0.6498791575431824</v>
       </c>
-      <c r="T51" t="n">
+      <c r="U51" t="n">
         <v>0.4661006927490234</v>
       </c>
-      <c r="U51" t="n">
+      <c r="V51" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="W51" t="n">
+        <v>0.3692358136177063</v>
+      </c>
+      <c r="X51" t="n">
         <v>3.681919</v>
       </c>
     </row>
@@ -4675,48 +5240,59 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Выпускникам', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Английский язык', 'Цифровые системы', 'Дополнительное образование']</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
           <t>Каникулярное время зависит от графика учебного процесса каждого учебного года. В 2024/2025 учебном году каникулы предоставляются до 12 августа. Если у вас есть дополнительные вопросы или требуется уточнение, пожалуйста, обращайтесь.  Подробнее: https://www.hse.ru/studyspravka/igaotpusk https://www.hse.ru/studyspravka/theend https://www.hse.ru/studyspravka/Otsrochka</t>
         </is>
       </c>
-      <c r="I52" t="n">
+      <c r="J52" t="n">
         <v>0</v>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>Последипломный отпуск Последипломный отпуск после прохождения студентами государственной итоговой аттестации Последипломные каникулы Процедура предоставления Документы Полезные ссылки ГИА (государственная итоговая аттестация) Сервис "Завершение обучения" График учебного процесса Приложение к диплому на английском языке После успешного прохождения государственной итоговой аттестации (далее — ГИА (государственная итоговая аттестация)) студенту могут быть предоставлены каникулы (последипломный отпуск). Продолжительность каникул определяется графиком учебного процесса текущего учебного года . В 2024/2025 уч. году каникулы предоставляются до 12 августа . Процедура предоставления каникул До начала ГИА (государственная итоговая аттестация) каждый студент, завершающий обучение, может подать заявку на последипломный отпуск в сервисе «Завершение обучения» Студенты, не подавшие заявления о предоставлении каникул, после успешного прохождения ГИА (государственная итоговая аттестация), подлежат отчислению из университета в связи с завершением обучения. В отношении студентов, подавших заявление о предоставлении каникул, издается приказ о предоставлении каникул (последипломного отпуска), дата заверш</t>
         </is>
       </c>
-      <c r="K52" t="n">
+      <c r="L52" t="n">
         <v>4</v>
       </c>
-      <c r="L52" t="n">
+      <c r="M52" t="n">
         <v>32</v>
       </c>
-      <c r="M52" t="n">
+      <c r="N52" t="n">
         <v>8</v>
       </c>
-      <c r="N52" t="n">
+      <c r="O52" t="n">
         <v>0.96875</v>
       </c>
-      <c r="O52" t="n">
+      <c r="P52" t="n">
         <v>0.1895810216665268</v>
       </c>
-      <c r="P52" t="n">
+      <c r="Q52" t="n">
         <v>0.05883798748254776</v>
       </c>
-      <c r="Q52" t="n">
+      <c r="R52" t="n">
         <v>0.751581072807312</v>
       </c>
-      <c r="R52" t="n">
+      <c r="S52" t="n">
         <v>16.7932542988229</v>
       </c>
-      <c r="S52" t="n">
+      <c r="T52" t="n">
         <v>0.5521530508995056</v>
       </c>
-      <c r="T52" t="n">
+      <c r="U52" t="n">
         <v>0.4914971590042114</v>
       </c>
-      <c r="U52" t="n">
+      <c r="V52" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="W52" t="n">
+        <v>0.4426033496856689</v>
+      </c>
+      <c r="X52" t="n">
         <v>3.480435</v>
       </c>
     </row>
@@ -4758,48 +5334,59 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Английский язык', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование', 'Социальные вопросы', 'Учебный процесс', 'ГИА', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Социальные вопросы', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Английский язык', 'Цифровые компетенции', 'Перемещения студентов / Изменения статусов студентов', 'Дополнительное образование']</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
           <t>Ваш индивидуальный учебный план (ИУП) доступен в электронной зачетке LMS НИУ ВШЭ (https://lms.hse.ru/index.php?page=gradebook).  Подробнее: https://www.hse.ru/docs/552116522.html https://www.hse.ru/studyspravka/plan https://www.hse.ru/docs/295301717.html</t>
         </is>
       </c>
-      <c r="I53" t="n">
+      <c r="J53" t="n">
         <v>1</v>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>Индивидуальный учебный план Индивидуальный учебный план (ИУП (индивидуальный учебный план)) Индивидуальный учебный план Что такое ИУП (индивидуальный учебный план) Как оформляется Где посмотреть свой ИУП (индивидуальный учебный план) Как внести изменения Специальный ИУП (индивидуальный учебный план) Документы Полезные ссылки Электронная зачетная книжка Кредит (зачетная единица) Контроль знаний студентов Перенос второй пересдачи дисциплины Отчисление Восстановление Что такое ИУП (индивидуальный учебный план) Индивидуальный учебный план (ИУП (индивидуальный учебный план)) — документ студента, в соответствии с которым он обязуется освоить элементы обучения (дисциплин/элементов практической подготовки) в определенный период. По каждому элементу ИУПа хранится информация о технологиях обучения, сроках изучения и прохождения промежуточной аттестации, объеме учебной нагрузки и основании включения этого элемента в учебный план. Для студентов большинства образовательных программ, ИУП (индивидуальный учебный план) составляется на полугодие, и все элементы, включенные в ИУП (индивидуальный учебный план), обязательны для освоения в этот период. Как ознакомиться со своим ИУП (индивидуальныйной программы и студентом; в течение трех рабочих дней после согласования ИУП (индивидуальный учебный план) готовит проект приказа о восстановлении студента/ допуске к учебным занятиям. Студент, который восстанавливается на место с коммерческой основой, стоимость оказываемых образовательных услуг не оплачивает. Заключение договора, не предусматривающего взимание платы, производится менеджером программы, на которую восстанавливается студент.</t>
         </is>
       </c>
-      <c r="K53" t="n">
+      <c r="L53" t="n">
         <v>1</v>
-      </c>
-      <c r="L53" t="n">
-        <v>13</v>
       </c>
       <c r="M53" t="n">
         <v>13</v>
       </c>
       <c r="N53" t="n">
+        <v>13</v>
+      </c>
+      <c r="O53" t="n">
         <v>1</v>
       </c>
-      <c r="O53" t="n">
+      <c r="P53" t="n">
         <v>0.5844770073890686</v>
       </c>
-      <c r="P53" t="n">
+      <c r="Q53" t="n">
         <v>0.2766598761081696</v>
       </c>
-      <c r="Q53" t="n">
+      <c r="R53" t="n">
         <v>0.138863131403923</v>
       </c>
-      <c r="R53" t="n">
+      <c r="S53" t="n">
         <v>4.873878063333527</v>
       </c>
-      <c r="S53" t="n">
+      <c r="T53" t="n">
         <v>0.462977409362793</v>
       </c>
-      <c r="T53" t="n">
+      <c r="U53" t="n">
         <v>0.4379397034645081</v>
       </c>
-      <c r="U53" t="n">
+      <c r="V53" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="W53" t="n">
+        <v>0.3981809318065643</v>
+      </c>
+      <c r="X53" t="n">
         <v>3.529985</v>
       </c>
     </row>
@@ -4841,48 +5428,59 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Обратная связь', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Учебный процесс', 'Цифровые системы', 'Обратная связь']</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
           <t>Да, студенческая оценка преподавания (СОП) является анонимной. Это значит, что студенты могут оставлять свои отзывы честно и подробно, а преподаватели и управленцы могут принимать решения на основе обобщенных данных, не зная, кто конкретно оставил тот или иной отзыв. Это позволяет сделать процесс обратной связи более открытым и эффективным.  Подробнее: https://www.hse.ru/studyspravka/evaluation\_prof http://www.hse.ru/evaluation/students\_mission https://www.hse.ru/evaluation/mustread https://www.hse.ru/evaluation/#timetable</t>
         </is>
       </c>
-      <c r="I54" t="n">
+      <c r="J54" t="n">
         <v>0</v>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>Студенческая оценка преподавания (СОП (студенческая оценка преподавания)) Студенческая оценка преподавания (СОП (студенческая оценка преподавания)): Информация для ППС Справочник преподавателя НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) Что такое СОП (студенческая оценка преподавания) Студенческая оценка преподавания (СОП (студенческая оценка преподавания)) – это ключевой для НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики) механизм сбора обратной связи об учебном процессе. СОП (студенческая оценка преподавания) помогает обеспечивать постоянное развитие качества преподавания и улучшение качества планирования и организации учебного процесса. СОП (студенческая оценка преподавания) проходит каждый модуль в течение последних 3 недель перед сессией. В анкете студентам предлагается оценить и прокомментировать качество преподавания и организации учебных дисциплин, высказать свои предложения по организации онлайн-курсов и проектной деятельности, а также — выразить свое мнение об организации учебного процесса на образовательной программе. → Подробнее о круге пользователей СОП (студенческая оценка преподавания), о блоках и особенностях анк помогает руководству оценивать учебный процесс на основе отзывов всех участников, а не только самых активных. Важно, что все ответы в СОП (студенческая оценка преподавания) анонимны — это позволяет студентам писать отзывы честно и подробно, а преподавателям и управленцам — выслушать всех и принять решения на обобщённых данных. СОП (студенческая оценка преподавания) проходит каждый модуль в последние 3 недели перед сессией. В анкете предлагается оценить и прокомментировать качество преподавания и организации учебных дисциплин, высказать свои предложения по организации онлайн-курсов и проектной деятельности, а еще — выразить свое мнение об организации учебного процесса на образовательной программе. С СОП (студенческая оценка преподавания) тесно связаны также механизмы оценки качества управления образовательным процессом и выборов лучших преподавателей (о них — ниже). Оценка качества управления образовательными программами Студенческая оценка качества управления образовательными программами (СОКУОП (студенческая оценка качества управления образовательными программами)) — ежегодный опрос, который проводится в конце 4-го модуля вместе с кампанией СОП (студенческая оценка преподавания). В СОКУОП (студенческая оценка качества управления образовательными программами) студсе и преподавателе. Вечерин Александр Викторович Академический руководитель ОП «Психология» (из материала для университетского издания « Окна роста » ) Руководители департаментов и кафедр Департаменты тоже получают данные СОП (студенческая оценка преподавания) по преподавателям — это помогает им оценить кадровый состав в их подразделении, подбирать кандидатуры преподавателей, а также в целом понимать, как развивать мастерство педагогического состава. СОП (студенческая оценка преподавания) в Школе иностранных языков глубоко встроена в бизнес-процессы и кадровую работу. У нас существует собственная кадровая комиссия, которая разрабатывает критерии оценки преподавательского мастерства вплоть до оценки занятий, мы создаём критерии к конкурсу ППС и мониторингу эффективности тьюторов, а ещё мы регулярно ходим на занятия к собственным преподавателям. В каждом из этих процессов мы используем СОП (студенческая оценка преподавания) в первую очередь для того, чтобы зафиксировать моменты, требующие корректировки — комментарии студентов часто показывают нам возможные проблемы в коммуникации, в проведении занятий, в оценке элементов контроля. И хотя обратная связь не всегда даёт полную информацию о происходящем на курсе, мы научились применять результаты анкетирования более глобально</t>
         </is>
       </c>
-      <c r="K54" t="n">
+      <c r="L54" t="n">
         <v>4</v>
       </c>
-      <c r="L54" t="n">
+      <c r="M54" t="n">
         <v>49</v>
       </c>
-      <c r="M54" t="n">
+      <c r="N54" t="n">
         <v>12.25</v>
       </c>
-      <c r="N54" t="n">
+      <c r="O54" t="n">
         <v>0.9183673469387755</v>
       </c>
-      <c r="O54" t="n">
+      <c r="P54" t="n">
         <v>0.9183480739593506</v>
       </c>
-      <c r="P54" t="n">
+      <c r="Q54" t="n">
         <v>0.04820806905627251</v>
       </c>
-      <c r="Q54" t="n">
+      <c r="R54" t="n">
         <v>0.03344390541315079</v>
       </c>
-      <c r="R54" t="n">
+      <c r="S54" t="n">
         <v>9.800995107875666</v>
       </c>
-      <c r="S54" t="n">
+      <c r="T54" t="n">
         <v>0.5917940735816956</v>
       </c>
-      <c r="T54" t="n">
+      <c r="U54" t="n">
         <v>0.490211695432663</v>
       </c>
-      <c r="U54" t="n">
+      <c r="V54" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="W54" t="n">
+        <v>0.2358916103839874</v>
+      </c>
+      <c r="X54" t="n">
         <v>32.817263</v>
       </c>
     </row>
@@ -4924,48 +5522,59 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Учебный процесс', 'Обратная связь', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Наука']</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
           <t>LMS (Learning management system) — это система поддержки очного и очно-заочного обучения, используемая в НИУ ВШЭ. Она предоставляет участникам учебного процесса доступ к материалам занятий, позволяет вести рабочую ведомость, обмениваться сообщениями, проводить тестирование и проверять знания студентов, а также сдавать проекты и домашние задания. Каждому студенту и преподавателю предоставляется доступ к SmartLMS по корпоративным учетным данным. Если возникают проблемы с подключением к системе, следует обратиться в Единое окно технической поддержки.  Подробнее: https://www.hse.ru/studyspravka/benefits https://www.hse.ru/studyspravka/lms https://www.hse.ru/studyspravka/zachetbook</t>
         </is>
       </c>
-      <c r="I55" t="n">
+      <c r="J55" t="n">
         <v>0</v>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t>Learning management system (LMS (Learning management system)) &amp; SmartLMS Learning management system (LMS (Learning management system)) &amp; SmartLMS SmartLMS SmartLMS — это единое образовательное пространство НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики), которое связывает всех участников учебного процесса. Образовательное пространство используется преподавателями для размещения материалов к занятиям, ведению рабочей ведомости, обмена сообщения со студентами, проведения тестирования для проверки полученных знаний промежуточного и итогового контроля, сдачи проектов и домашних заданий. SmartLMS доступна каждому студенту и преподавателю по корпоративным учетным данным (***@edu.hse.ru или ***@hse.ru) с авторизацией через Единый личный кабинет . Если у Вас возникли проблемы с подключением к системе, необходимо направить обращение в Единое окно технической поддержки . LMS (Learning management system) Learning Management System (LMS (Learning management system)) — система поддержки очного и очно-заочного обучения, которая используется всеми участниками учебного процесса. В LMS (Learning management system) у каждого студента есть возможность получить персонифицированную информацию об окончательных оценках по дисциплинам ( электронная зачетная книжка ), заполнить электронное портфолио студента , пройти студенческую оценку преподавания (СОП (студ</t>
         </is>
       </c>
-      <c r="K55" t="n">
+      <c r="L55" t="n">
         <v>5</v>
       </c>
-      <c r="L55" t="n">
+      <c r="M55" t="n">
         <v>71</v>
       </c>
-      <c r="M55" t="n">
+      <c r="N55" t="n">
         <v>14.2</v>
       </c>
-      <c r="N55" t="n">
+      <c r="O55" t="n">
         <v>0.8873239436619719</v>
       </c>
-      <c r="O55" t="n">
+      <c r="P55" t="n">
         <v>0.9881893396377563</v>
       </c>
-      <c r="P55" t="n">
+      <c r="Q55" t="n">
         <v>0.008498726412653923</v>
       </c>
-      <c r="Q55" t="n">
+      <c r="R55" t="n">
         <v>0.003311909269541502</v>
       </c>
-      <c r="R55" t="n">
+      <c r="S55" t="n">
         <v>36.13857166196545</v>
       </c>
-      <c r="S55" t="n">
+      <c r="T55" t="n">
         <v>0.7284385561943054</v>
       </c>
-      <c r="T55" t="n">
+      <c r="U55" t="n">
         <v>0.3196766972541809</v>
       </c>
-      <c r="U55" t="n">
+      <c r="V55" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="W55" t="n">
+        <v>0.248274177312851</v>
+      </c>
+      <c r="X55" t="n">
         <v>4.575349</v>
       </c>
     </row>
@@ -5007,48 +5616,59 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
+          <t>['Учебный процесс', 'Цифровые системы', 'Деньги', 'Учебный процесс', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Учебный процесс', 'Цифровые системы', 'Обратная связь', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы']</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
           <t>LMS (Learning management system) — это система поддержки очного и очно-заочного обучения, используемая в НИУ ВШЭ. Она предоставляет участникам учебного процесса доступ к материалам занятий, позволяет вести рабочую ведомость, обмениваться сообщениями, проводить тестирование и контроль знаний, а также сдавать проекты и домашние задания. LMS доступна каждому студенту и преподавателю по корпоративным учетным данным.  Подробнее: https://www.hse.ru/studyspravka/lms https://www.hse.ru/studyspravka/benefits https://www.hse.ru/studyspravka/zachetbook</t>
         </is>
       </c>
-      <c r="I56" t="n">
+      <c r="J56" t="n">
         <v>0</v>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>Learning management system (LMS (Learning management system)) &amp; SmartLMS Learning management system (LMS (Learning management system)) &amp; SmartLMS SmartLMS SmartLMS — это единое образовательное пространство НИУ (Национальный исследовательский университет) ВШЭ (Высшая школа экономики), которое связывает всех участников учебного процесса. Образовательное пространство используется преподавателями для размещения материалов к занятиям, ведению рабочей ведомости, обмена сообщения со студентами, проведения тестирования для проверки полученных знаний промежуточного и итогового контроля, сдачи проектов и домашних заданий. SmartLMS доступна каждому студенту и преподавателю по корпоративным учетным данным (***@edu.hse.ru или ***@hse.ru) с авторизацией через Единый личный кабинет . Если у Вас возникли проблемы с подключением к системе, необходимо направить обращение в Единое окно технической поддержки . LMS (Learning management system) Learning Management System (LMS (Learning management system)) — система поддержки очного и очно-заочного обучения, которая используется всеми участниками учебного процесса. В LMS (Learning management system) у каждого студента есть возможность получить персонифицированную информацию об окончательных оценках по дисциплинам ( электронная зачетная книжка ), заполнить электронное портфолио студента , пройти студенческую оценку преподавания (СОП (студ</t>
         </is>
       </c>
-      <c r="K56" t="n">
+      <c r="L56" t="n">
         <v>4</v>
       </c>
-      <c r="L56" t="n">
+      <c r="M56" t="n">
         <v>54</v>
       </c>
-      <c r="M56" t="n">
+      <c r="N56" t="n">
         <v>13.5</v>
       </c>
-      <c r="N56" t="n">
+      <c r="O56" t="n">
         <v>0.9259259259259259</v>
       </c>
-      <c r="O56" t="n">
+      <c r="P56" t="n">
         <v>0.8811179995536804</v>
       </c>
-      <c r="P56" t="n">
+      <c r="Q56" t="n">
         <v>0.110298790037632</v>
       </c>
-      <c r="Q56" t="n">
+      <c r="R56" t="n">
         <v>0.008583207614719868</v>
       </c>
-      <c r="R56" t="n">
+      <c r="S56" t="n">
         <v>30.6512955913039</v>
       </c>
-      <c r="S56" t="n">
+      <c r="T56" t="n">
         <v>0.702028751373291</v>
       </c>
-      <c r="T56" t="n">
+      <c r="U56" t="n">
         <v>0.2969781458377838</v>
       </c>
-      <c r="U56" t="n">
+      <c r="V56" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="W56" t="n">
+        <v>0.2680067420005798</v>
+      </c>
+      <c r="X56" t="n">
         <v>3.857499</v>
       </c>
     </row>
@@ -5090,48 +5710,59 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
+          <t>['Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Наука', 'Деньги', 'Учебный процесс', 'Практическая подготовка', 'Траектории обучения', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Наука', 'Учебный процесс', 'Практическая подготовка', 'ГИА', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Деньги', 'Учебный процесс', 'Перемещения студентов / Изменения статусов студентов', 'Цифровые системы', 'Социальные вопросы']</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
           <t>Даты сдачи курсовой работы устанавливаются факультетом и указываются в Порядке оформления курсовых и выпускных квалификационных работ. Обычно, студенты должны выбрать тему курсовой работы в установленные сроки. Если курсовая работа не сдана вовремя, это считается академической задолженностью и учитывается при расчете показателя качества учебной деятельности (КУД). Порядок ликвидации академической задолженности по курсовой работе включает в себя выполнение работы в установленный срок и ее успешную проверку. Информация о конкретных датах сдачи курсовой работы и порядке ликвидации задолженности обычно доступна в учебном офисе программы.  Подробнее: https://www.hse.ru/studyspravka/perezach https://www.hse.ru/studyspravka/instpaliat https://www.hse.ru/studyspravka/kursovrab https://www.hse.ru/studyspravka/vkr</t>
         </is>
       </c>
-      <c r="I57" t="n">
+      <c r="J57" t="n">
         <v>0</v>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t>обязанностей по добросовестному освоению ОП. * В отдельных случаях ОП может устанавливать свои периоды предложения и выбора тем КР (курсовая работа). С более подробной информацией можно ознакомиться в программе практики на сайте ОП или уточнить в учебном офисе. Что будет, если не сдать курсовую работу в установленный срок? Невыполнение работы в установленный факультетом срок считается академической задолженностью и учитывается в расчете показателя качества учебной деятельности (КУД (качество учебной деятельности)). Подробнее о расчете КУД (качество учебной деятельности) и ликвидации задолженности — в ПОПАТКУС (Положения о промежуточной аттестации и текущем контроле успеваемости студентов) . Каков порядок ликвидации академической задолженности по курсовой работе? Академическая задолженность по курсовой работе наступает в случае: невыполнения работы в установленный факультетом срок (работа не сдана в установленном порядке и (или) не загружена в систему LMS (Learning management system) для проверки в системе "Антиплагиат"); выявления в работе заимствований, ставящих под сомнение самостоятельность выполнения работы (следствием может быть дисциплинарное взыскание в виде отчисления); получения неудовлетворительной оценки, неявки на защиту (ат". По итогам проверки в карточке работы отображается следующая информация: Тема работы на русском Тема на английском Дата загрузки Процент плагиата Статус о завершении проверки Дополнительно формируется QR-код в формате pdf, который служит подтверждением загрузки работы в систему LMS (Learning management system) и проверкой на плагиат. QR-код необходимо предоставить вместе с выпускной квалификационной работой и отзывом научного руководителя в порядке, установленном образовательной программой (срок, место сдачи работы) Нашли опечатку ? Выделите её, нажмите Ctrl+Enter и отправьте нам уведомление. Спасибо за участие! Сервис предназначен только для отправки сообщений об орфографических и пунктуационных ошибках.</t>
         </is>
       </c>
-      <c r="K57" t="n">
+      <c r="L57" t="n">
         <v>6</v>
       </c>
-      <c r="L57" t="n">
+      <c r="M57" t="n">
         <v>82</v>
       </c>
-      <c r="M57" t="n">
+      <c r="N57" t="n">
         <v>13.66666666666667</v>
       </c>
-      <c r="N57" t="n">
+      <c r="O57" t="n">
         <v>0.7560975609756098</v>
       </c>
-      <c r="O57" t="n">
+      <c r="P57" t="n">
         <v>0.7080943584442139</v>
       </c>
-      <c r="P57" t="n">
+      <c r="Q57" t="n">
         <v>0.1115799993276596</v>
       </c>
-      <c r="Q57" t="n">
+      <c r="R57" t="n">
         <v>0.1803256869316101</v>
       </c>
-      <c r="R57" t="n">
+      <c r="S57" t="n">
         <v>30.39826939802096</v>
       </c>
-      <c r="S57" t="n">
+      <c r="T57" t="n">
         <v>0.6521539688110352</v>
       </c>
-      <c r="T57" t="n">
+      <c r="U57" t="n">
         <v>0.4309975504875183</v>
       </c>
-      <c r="U57" t="n">
+      <c r="V57" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="W57" t="n">
+        <v>0.3610856533050537</v>
+      </c>
+      <c r="X57" t="n">
         <v>3.860324</v>
       </c>
     </row>

</xml_diff>